<commit_message>
Map Adapter_Order from a single SAPI field per target column.
SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID,
CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY,
TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID empty. Currency KES.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -93,6 +98,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -560,7 +568,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Order</t>
@@ -586,14 +594,192 @@
           <t>dwl/map-adapter-order.dwl</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 154,
+      "ENTRY_ID": 60,
+      "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1701,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "FAVOUR SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 89,
+      "PRODUCT_REF": "BIC976044",
+      "PRODUCT_CODE": "BIC976044",
+      "PRODUCT_CATEGORY": "SHAVERS",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
+      "PACKAGING": "PIECE",
+      "QUANTITY": 96,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 22.85,
+      "SELLING_PRICE": 22.67,
+      "VALUE_SOLD": 2176.32,
+      "SALES_VALUE": 1876.137931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T14:03:22",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T14:03:24",
+      "UPDATED_AT": "2026-08-20T14:03:24",
+      "DISCOUNT": 17.28,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 22.67,
+      "PRICE_VAT_EXC": 19.543103,
+      "PRICE_VAT": 3.1268965517,
+      "TOTAL_VAT_INC": 2176.32,
+      "TOTAL_VAT_EXC": 1876.137931,
+      "TOTAL_VAT": 300.1820689655,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T14:02:14",
+      "CHECKOUTTIME": "2026-08-20T14:03:24"
+    },
+    {
+      "ID": 153,
+      "ENTRY_ID": 59,
+      "VISIT_ID": "2e96e08a-19e3-4f6a-ab11-3c9a10d28bdf",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1704,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "MOLLYS SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:56:17",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 8,
+      "PRODUCT_REF": "BIC301209",
+      "PRODUCT_CODE": "BIC301209",
+      "PRODUCT_CATEGORY": "STATIONERY",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "CRISTAL MED BLU BX 25 LB KE",
+      "PACKAGING": "PACKET",
+      "QUANTITY": 2,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 372,
+      "SELLING_PRICE": 372,
+      "VALUE_SOLD": 744,
+      "SALES_VALUE": 641.37931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T13:38:36",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T13:38:38",
+      "UPDATED_AT": "2026-08-20T13:38:38",
+      "DISCOUNT": 0,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 372,
+      "PRICE_VAT_EXC": 320.689655,
+      "PRICE_VAT": 51.3103448276,
+      "TOTAL_VAT_INC": 744,
+      "TOTAL_VAT_EXC": 641.37931,
+      "TOTAL_VAT": 102.6206896552,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T13:37:17",
+      "CHECKOUTTIME": "2026-08-20T13:38:39"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 1701,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC976044",
+      "DistributorID": "",
+      "WarehouseID": 183,
+      "OrderNumber": 60,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "14:02:14",
+      "OrderEndTime": "14:03:24",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PIECE",
+      "Currency": "KES",
+      "QuantityOrdered": 96,
+      "AmountOrdered": 2176.32,
+      "Discount": 17.28,
+      "VATAmount": 300.1820689655
+    },
+    {
+      "StoreID": 1704,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC301209",
+      "DistributorID": "",
+      "WarehouseID": 183,
+      "OrderNumber": 59,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "13:37:17",
+      "OrderEndTime": "13:38:39",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PACKET",
+      "Currency": "KES",
+      "QuantityOrdered": 2,
+      "AmountOrdered": 744,
+      "Discount": 0,
+      "VATAmount": 102.6206896552
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID empty. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1276,7 +1462,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>SHOP_ID / SHOPID</t>
+          <t>SHOP_ID</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1320,7 +1506,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>routeid / ROUTEID</t>
+          <t>ROUTEID</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1347,7 +1533,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is (no letter strip)</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1550,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(property / empty)</t>
+          <t>(empty)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>papi.sat.solutech.distributor.id</t>
+          <t>constant empty until value known</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1572,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>supplier_id / SUPPLIER_ID</t>
+          <t>SUPPLIER_ID</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update mapping workbook with Order SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -93,6 +98,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,7 +469,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -560,7 +568,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Order</t>
@@ -586,14 +594,192 @@
           <t>dwl/map-adapter-order.dwl</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 154,
+      "ENTRY_ID": 60,
+      "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1701,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "FAVOUR SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 89,
+      "PRODUCT_REF": "BIC976044",
+      "PRODUCT_CODE": "BIC976044",
+      "PRODUCT_CATEGORY": "SHAVERS",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
+      "PACKAGING": "PIECE",
+      "QUANTITY": 96,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 22.85,
+      "SELLING_PRICE": 22.67,
+      "VALUE_SOLD": 2176.32,
+      "SALES_VALUE": 1876.137931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T14:03:22",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T14:03:24",
+      "UPDATED_AT": "2026-08-20T14:03:24",
+      "DISCOUNT": 17.28,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 22.67,
+      "PRICE_VAT_EXC": 19.543103,
+      "PRICE_VAT": 3.1268965517,
+      "TOTAL_VAT_INC": 2176.32,
+      "TOTAL_VAT_EXC": 1876.137931,
+      "TOTAL_VAT": 300.1820689655,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T14:02:14",
+      "CHECKOUTTIME": "2026-08-20T14:03:24"
+    },
+    {
+      "ID": 153,
+      "ENTRY_ID": 59,
+      "VISIT_ID": "2e96e08a-19e3-4f6a-ab11-3c9a10d28bdf",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1704,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "MOLLYS SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:56:17",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 8,
+      "PRODUCT_REF": "BIC301209",
+      "PRODUCT_CODE": "BIC301209",
+      "PRODUCT_CATEGORY": "STATIONERY",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "CRISTAL MED BLU BX 25 LB KE",
+      "PACKAGING": "PACKET",
+      "QUANTITY": 2,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 372,
+      "SELLING_PRICE": 372,
+      "VALUE_SOLD": 744,
+      "SALES_VALUE": 641.37931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T13:38:36",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T13:38:38",
+      "UPDATED_AT": "2026-08-20T13:38:38",
+      "DISCOUNT": 0,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 372,
+      "PRICE_VAT_EXC": 320.689655,
+      "PRICE_VAT": 51.3103448276,
+      "TOTAL_VAT_INC": 744,
+      "TOTAL_VAT_EXC": 641.37931,
+      "TOTAL_VAT": 102.6206896552,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T13:37:17",
+      "CHECKOUTTIME": "2026-08-20T13:38:39"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 1701,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC976044",
+      "DistributorID": "",
+      "WarehouseID": 183,
+      "OrderNumber": 60,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "14:02:14",
+      "OrderEndTime": "14:03:24",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PIECE",
+      "Currency": "KES",
+      "QuantityOrdered": 96,
+      "AmountOrdered": 2176.32,
+      "Discount": 17.28,
+      "VATAmount": 300.1820689655
+    },
+    {
+      "StoreID": 1704,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC301209",
+      "DistributorID": "",
+      "WarehouseID": 183,
+      "OrderNumber": 59,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "13:37:17",
+      "OrderEndTime": "13:38:39",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PACKET",
+      "Currency": "KES",
+      "QuantityOrdered": 2,
+      "AmountOrdered": 744,
+      "Discount": 0,
+      "VATAmount": 102.6206896552
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID empty. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -837,7 +1023,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D64"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -1276,7 +1462,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>SHOP_ID / SHOPID</t>
+          <t>SHOP_ID</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1320,7 +1506,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>routeid / ROUTEID</t>
+          <t>ROUTEID</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1347,7 +1533,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is (no letter strip)</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1550,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(property / empty)</t>
+          <t>(empty)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>papi.sat.solutech.distributor.id</t>
+          <t>constant empty until value known</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1572,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>supplier_id / SUPPLIER_ID</t>
+          <t>SUPPLIER_ID</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2265,7 +2451,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Map Adapter_Product from one SAPI field per column.
productcode to ProductID from first numeric, product_desc to ProductSKU, uomname to UnitofMeasure.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -781,7 +781,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="220" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Product</t>
@@ -807,14 +807,112 @@
           <t>dwl/map-adapter-product.dwl</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "productcode": "BIC502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    },
+    {
+      "id": 2,
+      "productcode": "BIC502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "ProductID": "502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    },
+    {
+      "id": 2,
+      "ProductID": "502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1863,7 +1961,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>strip leading letters (BIC502418 → 502418)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update mapping workbook with Product SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -781,7 +781,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="220" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Product</t>
@@ -807,14 +807,112 @@
           <t>dwl/map-adapter-product.dwl</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "productcode": "BIC502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    },
+    {
+      "id": 2,
+      "productcode": "BIC502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "ProductID": "502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    },
+    {
+      "id": 2,
+      "ProductID": "502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1863,7 +1961,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>strip leading letters (BIC502418 → 502418)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Map Adapter_Route from one SAPI field per column.
route_id, route_name, userid, visit_frequency, saler_category, created_at as Date.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,6 +101,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -914,7 +917,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="180" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Route</t>
@@ -940,16 +943,82 @@
           <t>dwl/map-adapter-route.dwl</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 31,
+      "route_id": 31,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "DICKSON NJUE MONDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:15:47",
+      "updated_at": "2026-06-15T11:15:47",
+      "userid": 75,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "MON",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    },
+    {
+      "id": 33,
+      "route_id": 33,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "PHILIP DAVID TUESDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:19:06",
+      "updated_at": "2026-06-15T11:19:06",
+      "userid": 73,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "TUE",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "RouteID": 31,
+      "RouteName": "DICKSON NJUE MONDAY",
+      "SalesRepID": 75,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    },
+    {
+      "RouteID": 33,
+      "RouteName": "PHILIP DAVID TUESDAY",
+      "SalesRepID": 73,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2320,39 +2389,39 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>RouteID</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>route_id</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>RouteName</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>route_name</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2364,17 +2433,17 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>SalesRepID</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>userid</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2386,39 +2455,39 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>RouteType</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>visit_frequency</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>SalesRepType</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>saler_category</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2430,108 +2499,218 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>dd/MM/yyyy</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>ProductID</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>routes.* + userid, visit_frequency, visit_week, visit_day, status, saler_category</t>
+          <t>productcode</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>strip leading letters</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>SalesRep</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>UnitofMeasure</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>users.* + saler_category</t>
+          <t>UOMName</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseName</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>stockpoint_name</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>SalesRep</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>users.* + saler_category</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>customers.*</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Update mapping workbook with Route SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,6 +101,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -914,7 +917,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="180" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Route</t>
@@ -940,16 +943,82 @@
           <t>dwl/map-adapter-route.dwl</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 31,
+      "route_id": 31,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "DICKSON NJUE MONDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:15:47",
+      "updated_at": "2026-06-15T11:15:47",
+      "userid": 75,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "MON",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    },
+    {
+      "id": 33,
+      "route_id": 33,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "PHILIP DAVID TUESDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:19:06",
+      "updated_at": "2026-06-15T11:19:06",
+      "userid": 73,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "TUE",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "RouteID": 31,
+      "RouteName": "DICKSON NJUE MONDAY",
+      "SalesRepID": 75,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    },
+    {
+      "RouteID": 33,
+      "RouteName": "PHILIP DAVID TUESDAY",
+      "SalesRepID": 73,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2320,39 +2389,39 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>RouteID</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>route_id</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>RouteName</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>route_name</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2364,17 +2433,17 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>SalesRepID</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>userid</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2386,39 +2455,39 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>RouteType</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>visit_frequency</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>SalesRepType</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>saler_category</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2430,108 +2499,218 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>dd/MM/yyyy</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>ProductID</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>routes.* + userid, visit_frequency, visit_week, visit_day, status, saler_category</t>
+          <t>productcode</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>strip leading letters</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>SalesRep</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>UnitofMeasure</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>users.* + saler_category</t>
+          <t>UOMName</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseName</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>stockpoint_name</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>SalesRep</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>users.* + saler_category</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>customers.*</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Map Adapter_SalesRep from one SAPI field per column.
id, name, warehouse_code, saler_category. DistributorID empty.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1022,7 +1022,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>SalesRep</t>
@@ -1048,16 +1048,90 @@
           <t>dwl/map-adapter-salesrep.dwl</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 72,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 4,
+      "name": "ESTHER KAGIRI",
+      "email": "ngong@nobleoutlook.co.ke",
+      "phone_number": "0710000000",
+      "last_time_active": "3",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Inactive",
+      "territory_id": null,
+      "rolegroup_id": 4,
+      "vehicle_id": 4,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:40:33",
+      "saler_category": "Drivers (Delivery Agents)"
+    },
+    {
+      "id": 73,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 5,
+      "name": "PHILLIP DAVID",
+      "email": "ngong1@nobleoutlook.co.ke",
+      "phone_number": "0710000001",
+      "last_time_active": "5",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Active",
+      "territory_id": null,
+      "rolegroup_id": 5,
+      "vehicle_id": 2,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:44:40",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "SalesRepID": 72,
+      "SalesRepName": "ESTHER KAGIRI",
+      "DistributorID": "",
+      "WarehouseID": "",
+      "SalesRepType": "Drivers (Delivery Agents)"
+    },
+    {
+      "SalesRepID": 73,
+      "SalesRepName": "PHILLIP DAVID",
+      "DistributorID": "",
+      "WarehouseID": "",
+      "SalesRepType": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>id, name, warehouse_code, saler_category. DistributorID empty. One field each.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2521,39 +2595,39 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>SalesRepID</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>SalesRepName</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2565,61 +2639,61 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>DistributorID</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>(empty)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>constant empty until value known</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>warehouse_code</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>SalesRepType</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>saler_category</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -2636,81 +2710,169 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>ProductID</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>productcode</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>strip leading letters</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SalesRep</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>UnitofMeasure</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>users.* + saler_category</t>
+          <t>UOMName</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseName</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>stockpoint_name</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>customers.*</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Update mapping workbook with SalesRep SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1022,7 +1022,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>SalesRep</t>
@@ -1048,16 +1048,90 @@
           <t>dwl/map-adapter-salesrep.dwl</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 72,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 4,
+      "name": "ESTHER KAGIRI",
+      "email": "ngong@nobleoutlook.co.ke",
+      "phone_number": "0710000000",
+      "last_time_active": "3",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Inactive",
+      "territory_id": null,
+      "rolegroup_id": 4,
+      "vehicle_id": 4,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:40:33",
+      "saler_category": "Drivers (Delivery Agents)"
+    },
+    {
+      "id": 73,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 5,
+      "name": "PHILLIP DAVID",
+      "email": "ngong1@nobleoutlook.co.ke",
+      "phone_number": "0710000001",
+      "last_time_active": "5",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Active",
+      "territory_id": null,
+      "rolegroup_id": 5,
+      "vehicle_id": 2,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:44:40",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "SalesRepID": 72,
+      "SalesRepName": "ESTHER KAGIRI",
+      "DistributorID": "",
+      "WarehouseID": "",
+      "SalesRepType": "Drivers (Delivery Agents)"
+    },
+    {
+      "SalesRepID": 73,
+      "SalesRepName": "PHILLIP DAVID",
+      "DistributorID": "",
+      "WarehouseID": "",
+      "SalesRepType": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>id, name, warehouse_code, saler_category. DistributorID empty. One field each.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2521,39 +2595,39 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>SalesRepID</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>SalesRepName</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2565,61 +2639,61 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>DistributorID</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>(empty)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>constant empty until value known</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>warehouse_code</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>SalesRep</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>SalesRepType</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>saler_category</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -2636,81 +2710,169 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>ProductID</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>productcode</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>strip leading letters</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SalesRep</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>UnitofMeasure</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>users.* + saler_category</t>
+          <t>UOMName</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseName</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>stockpoint_name</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>(SAPI columns as-is)</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>customers.*</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>pass-through until payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Set DistributorID to ??? for Order and SalesRep mappings.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -741,7 +741,7 @@
       "SalesRepID": "THOMAS OUMA",
       "RouteID": 85,
       "ProductID": "BIC976044",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": 183,
       "OrderNumber": 60,
       "OrderDate": "20/08/2026",
@@ -760,7 +760,7 @@
       "SalesRepID": "THOMAS OUMA",
       "RouteID": 85,
       "ProductID": "BIC301209",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": 183,
       "OrderNumber": 59,
       "OrderDate": "20/08/2026",
@@ -780,7 +780,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID empty. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
         </is>
       </c>
     </row>
@@ -1114,14 +1114,14 @@
     {
       "SalesRepID": 72,
       "SalesRepName": "ESTHER KAGIRI",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": "",
       "SalesRepType": "Drivers (Delivery Agents)"
     },
     {
       "SalesRepID": 73,
       "SalesRepName": "PHILLIP DAVID",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": "",
       "SalesRepType": "Van Sales"
     }
@@ -1131,7 +1131,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>id, name, warehouse_code, saler_category. DistributorID empty. One field each.</t>
+          <t>id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
         </is>
       </c>
     </row>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(empty)</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>constant empty until value known</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>
@@ -2649,12 +2649,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>(empty)</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>constant empty until value known</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Order and SalesRep DistributorID to ??? in the workbook.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -741,7 +741,7 @@
       "SalesRepID": "THOMAS OUMA",
       "RouteID": 85,
       "ProductID": "BIC976044",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": 183,
       "OrderNumber": 60,
       "OrderDate": "20/08/2026",
@@ -760,7 +760,7 @@
       "SalesRepID": "THOMAS OUMA",
       "RouteID": 85,
       "ProductID": "BIC301209",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": 183,
       "OrderNumber": 59,
       "OrderDate": "20/08/2026",
@@ -780,7 +780,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID empty. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
         </is>
       </c>
     </row>
@@ -1114,14 +1114,14 @@
     {
       "SalesRepID": 72,
       "SalesRepName": "ESTHER KAGIRI",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": "",
       "SalesRepType": "Drivers (Delivery Agents)"
     },
     {
       "SalesRepID": 73,
       "SalesRepName": "PHILLIP DAVID",
-      "DistributorID": "",
+      "DistributorID": "???",
       "WarehouseID": "",
       "SalesRepType": "Van Sales"
     }
@@ -1131,7 +1131,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>id, name, warehouse_code, saler_category. DistributorID empty. One field each.</t>
+          <t>id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
         </is>
       </c>
     </row>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(empty)</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>constant empty until value known</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>
@@ -2649,12 +2649,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>(empty)</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>constant empty until value known</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Map Adapter_Customer from one SAPI field per column.
CHANNEL to Channel and StoreClassification. WarehouseID is ???.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1135,7 +1135,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Customer</t>
@@ -1161,16 +1161,156 @@
           <t>dwl/map-adapter-customer.dwl</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 199,
+      "SHOPID": 199,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "MANDELA SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254722590524",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "IAN MWENDWA",
+      "VERIFIEDDATE": "2026-06-15T14:35:26",
+      "ADDEDBY": "PHILLIP DAVID",
+      "USERID": 73,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "PINCH ANISO",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:27:43",
+      "LASTSALE": "2026-06-15T15:07:50",
+      "LATITUDE": -1.2349905,
+      "LONGITUDE": 36.9328219,
+      "DATECREATED": "2026-06-15T14:17:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    },
+    {
+      "ID": 200,
+      "SHOPID": 200,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "GB SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254725446821",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "CLEMENCEA SARU",
+      "VERIFIEDDATE": "2026-06-15T16:09:14",
+      "ADDEDBY": "DICKSON NJUE",
+      "USERID": 75,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "GB",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:28:04",
+      "LASTSALE": "2026-08-31T17:08:17",
+      "LATITUDE": -1.2562547,
+      "LONGITUDE": 36.9237899,
+      "DATECREATED": "2026-06-15T16:07:17",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 199,
+      "StoreName": "MANDELA SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9328219,
+      "Latitude": -1.2349905,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    },
+    {
+      "StoreID": 200,
+      "StoreName": "GB SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9237899,
+      "Latitude": -1.2562547,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>SAPI path is /api/store until Exchange adds /api/customer.</t>
+          <t>CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2705,39 +2845,39 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>StoreID</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>SHOPID</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>StoreName</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>CUSTOMERNAME</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -2749,17 +2889,17 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>StoreCategory</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>CUSTOMERCATEGORY</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -2771,66 +2911,66 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>CHANNEL</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>StoreClassification</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>CHANNEL</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>same as Channel</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>
@@ -2842,37 +2982,323 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>LONGITUDE</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>LATITUDE</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>LOCATIONNAME</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>REGIONNAME</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>StoreStatus</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>StoreCreationDate</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>DATECREATED</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>StoreSize</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>ProductID</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>productcode</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>strip leading letters</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>UnitofMeasure</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>UOMName</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>WarehouseName</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>stockpoint_name</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Update mapping workbook with Customer SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1135,7 +1135,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Customer</t>
@@ -1161,16 +1161,156 @@
           <t>dwl/map-adapter-customer.dwl</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 199,
+      "SHOPID": 199,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "MANDELA SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254722590524",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "IAN MWENDWA",
+      "VERIFIEDDATE": "2026-06-15T14:35:26",
+      "ADDEDBY": "PHILLIP DAVID",
+      "USERID": 73,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "PINCH ANISO",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:27:43",
+      "LASTSALE": "2026-06-15T15:07:50",
+      "LATITUDE": -1.2349905,
+      "LONGITUDE": 36.9328219,
+      "DATECREATED": "2026-06-15T14:17:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    },
+    {
+      "ID": 200,
+      "SHOPID": 200,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "GB SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254725446821",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "CLEMENCEA SARU",
+      "VERIFIEDDATE": "2026-06-15T16:09:14",
+      "ADDEDBY": "DICKSON NJUE",
+      "USERID": 75,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "GB",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:28:04",
+      "LASTSALE": "2026-08-31T17:08:17",
+      "LATITUDE": -1.2562547,
+      "LONGITUDE": 36.9237899,
+      "DATECREATED": "2026-06-15T16:07:17",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 199,
+      "StoreName": "MANDELA SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9328219,
+      "Latitude": -1.2349905,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    },
+    {
+      "StoreID": 200,
+      "StoreName": "GB SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9237899,
+      "Latitude": -1.2562547,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>SAPI path is /api/store until Exchange adds /api/customer.</t>
+          <t>CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2705,39 +2845,39 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>StoreID</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>productcode</t>
+          <t>SHOPID</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>UnitofMeasure</t>
+          <t>StoreName</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>CUSTOMERNAME</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -2749,17 +2889,17 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>StoreCategory</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>stockpoint_name</t>
+          <t>CUSTOMERCATEGORY</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -2771,66 +2911,66 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>date_created</t>
+          <t>CHANNEL</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>StoreClassification</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>CHANNEL</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>same as Channel</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>total_cost</t>
+          <t>(literal ???)</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>constant "???"</t>
         </is>
       </c>
     </row>
@@ -2842,37 +2982,323 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>customers.*</t>
+          <t>LONGITUDE</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>LATITUDE</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>LOCATIONNAME</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>REGIONNAME</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>StoreStatus</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>StoreCreationDate</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>DATECREATED</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>StoreSize</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>ProductID</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>productcode</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>strip leading letters</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>UnitofMeasure</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>UOMName</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>WarehouseName</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>stockpoint_name</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>DateCreated</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>date_created</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>dd/MM/yyyy</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>TotalCost</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>(SAPI columns as-is)</t>
         </is>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>customers.* where CUSTOMER_TYPE=Supplier</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>pass-through until payload</t>
         </is>

</xml_diff>

<commit_message>
Map Adapter_Stock from one SAPI field per column.
productcode to ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1314,7 +1314,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="180" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Stock</t>
@@ -1340,16 +1340,62 @@
           <t>dwl/map-adapter-stock.dwl</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": null,
+      "date_created": "2026-08-17T14:00:56",
+      "quantity": 2640,
+      "total_cost": 1060
+    },
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": "GIKAMBURA STOCKPOINT",
+      "date_created": "2026-08-14T12:42:33",
+      "quantity": 2640,
+      "total_cost": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "",
+      "Date": "17/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1060
+    },
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "GIKAMBURA STOCKPOINT",
+      "Date": "14/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>SAPI path is /api/inventory until Exchange adds /api/stock.</t>
+          <t>productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3204,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>ProductSKU</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -3168,7 +3214,7 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>from first numeric (BIC969584 → 969584)</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3231,7 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>uomname</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -3202,7 +3248,7 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>DistributorWarehouseCode</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -3224,7 +3270,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -3246,7 +3292,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>InventoryQuantity</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -3268,7 +3314,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>InventoryPrice</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update mapping workbook with Stock SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1314,7 +1314,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="180" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Stock</t>
@@ -1340,16 +1340,62 @@
           <t>dwl/map-adapter-stock.dwl</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": null,
+      "date_created": "2026-08-17T14:00:56",
+      "quantity": 2640,
+      "total_cost": 1060
+    },
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": "GIKAMBURA STOCKPOINT",
+      "date_created": "2026-08-14T12:42:33",
+      "quantity": 2640,
+      "total_cost": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "",
+      "Date": "17/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1060
+    },
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "GIKAMBURA STOCKPOINT",
+      "Date": "14/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>SAPI path is /api/inventory until Exchange adds /api/stock.</t>
+          <t>productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3204,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>ProductID</t>
+          <t>ProductSKU</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -3168,7 +3214,7 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>from first numeric (BIC969584 → 969584)</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3231,7 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>UOMName</t>
+          <t>uomname</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -3202,7 +3248,7 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>WarehouseName</t>
+          <t>DistributorWarehouseCode</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -3224,7 +3270,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>DateCreated</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -3246,7 +3292,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>InventoryQuantity</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -3268,7 +3314,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>TotalCost</t>
+          <t>InventoryPrice</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Map Adapter_Warehouse from one SAPI field per column.
ID to WarehouseID, CUSTOMERNAME to WarehouseName, DistributorID empty.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1399,7 +1399,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="180" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Warehouse</t>
@@ -1425,16 +1425,134 @@
           <t>dwl/map-adapter-warehouse.dwl</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 183,
+      "SHOPID": 183,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "183",
+      "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 4,
+      "LOCATIONNAME": "GIKAMBURA",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Pending",
+      "VERIFIEDBY": null,
+      "VERIFIEDDATE": null,
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-08T15:07:59",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    },
+    {
+      "ID": 186,
+      "SHOPID": 186,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "186",
+      "CUSTOMERNAME": "NAIROBI WEST STCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 1,
+      "LOCATIONNAME": "NAIROBI WEST",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "TECLA AYORE",
+      "VERIFIEDDATE": "2026-06-09T22:46:16",
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-09T22:42:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "WarehouseID": 183,
+      "WarehouseName": "GIKAMBURA STOCKPOINT",
+      "DistributorID": ""
+    },
+    {
+      "WarehouseID": 186,
+      "WarehouseName": "NAIROBI WEST STCKPOINT",
+      "DistributorID": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each.</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3336,17 +3454,61 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>customers.* where CUSTOMER_TYPE=Supplier</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>WarehouseName</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>CUSTOMERNAME</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>DistributorID</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update mapping workbook with Warehouse SAPI and PAPI payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1399,7 +1399,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="180" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Warehouse</t>
@@ -1425,16 +1425,134 @@
           <t>dwl/map-adapter-warehouse.dwl</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>WAITING — currently pass-through</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 183,
+      "SHOPID": 183,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "183",
+      "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 4,
+      "LOCATIONNAME": "GIKAMBURA",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Pending",
+      "VERIFIEDBY": null,
+      "VERIFIEDDATE": null,
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-08T15:07:59",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    },
+    {
+      "ID": 186,
+      "SHOPID": 186,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "186",
+      "CUSTOMERNAME": "NAIROBI WEST STCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 1,
+      "LOCATIONNAME": "NAIROBI WEST",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "TECLA AYORE",
+      "VERIFIEDDATE": "2026-06-09T22:46:16",
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-09T22:42:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "WarehouseID": 183,
+      "WarehouseName": "GIKAMBURA STOCKPOINT",
+      "DistributorID": ""
+    },
+    {
+      "WarehouseID": 186,
+      "WarehouseName": "NAIROBI WEST STCKPOINT",
+      "DistributorID": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>PAPI currently returns SAPI columns as-is.</t>
+          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each.</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3336,17 +3454,61 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>(SAPI columns as-is)</t>
+          <t>WarehouseID</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>customers.* where CUSTOMER_TYPE=Supplier</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>pass-through until payload</t>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>WarehouseName</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>CUSTOMERNAME</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>DistributorID</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>(hardcoded empty)</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>constant empty</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep Exp GET /v1/Customer and /v1/Stock and drop Store and Inventory aliases.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1143,7 +1143,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>/api/store (Customer SQL)</t>
+          <t>/api/customer</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/Store (or /v1/Customer after RAML)</t>
+          <t>/api/v1/Customer</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>/api/inventory (Stock SQL)</t>
+          <t>/api/stock</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/Inventory (or /v1/Stock after RAML)</t>
+          <t>/api/v1/Stock</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each.</t>
+          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Call SAPI /api/customer and /api/stock from Adapter_Customer and Adapter_Stock.
Remove store and inventory path aliases. Update Postman and the mapping workbook to the same names.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1143,7 +1143,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>/api/store (Customer SQL)</t>
+          <t>/api/customer</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/Store (or /v1/Customer after RAML)</t>
+          <t>/api/v1/Customer</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>/api/inventory (Stock SQL)</t>
+          <t>/api/stock</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/Inventory (or /v1/Stock after RAML)</t>
+          <t>/api/v1/Stock</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each.</t>
+          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put SAPI payload, transformed payload, and mapping as the first three Excel columns.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -7,11 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Endpoints" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current field map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="How this sheet is filled" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Payloads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Endpoints" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Current field map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How this sheet is filled" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Payloads'!$A$1:$I$9</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -32,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,8 +62,13 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -82,11 +90,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -104,6 +126,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,18 +502,18 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Resource</t>
@@ -493,116 +521,109 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>SAPI payload</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Transformed payload</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mapping</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>SAPI endpoint</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PAPI endpoint</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Exp (EAPI) endpoint</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Exp endpoint</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAPI mapping file</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Mapping status</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SAPI payload (paste)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Final payload after PAPI mapping</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr"/>
+      <c r="C2" s="7" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>STOREID ← SHOPID
+Discount ← DISCOUNT
+SalesRepID ← USERID
+VATAmount ← TOTAL_VAT
+RouteID ← ROUTEID
+DistributorID ← (property / empty)  (papi.sat.solutech.distributor.id)
+ProductID ← PRODUCT_CODE  (strip leading letters)
+WarehouseID ← SUPPLIER_ID
+OrderNumber ← SALE_ORDER_ID
+InvoiceNumber ← ENTRY_ID
+InvoiceDate ← CREATED_AT  (dd/MM/yyyy)
+InvoiceTime ← CREATED_AT  (HH:mm:ss)
+InvoiceStatus ← PAYMENT_STATUS
+UnitOfMeasure ← PACKAGING
+Currency ← (constant)  (KES)
+QuantityInvoiced ← QUANTITY
+AmountInvoiced ← VALUE_SOLD
+TransType ← ENTRY_TYPE
+Notes: Invoice mapping already live. Do not change until you paste SAPI payload.</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>/api/invoice</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>/api/Adapter_Invoice</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>/api/v1/Invoice</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>dwl/map-adapter-invoice.dwl</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>WAITING for real SAPI payload</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Invoice mapping already live. Do not change until you paste SAPI payload.</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="220" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>/api/order</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Order</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Order</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-order.dwl</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -732,7 +753,7 @@
 }</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -778,44 +799,61 @@
 }</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>StoreID ← SHOP_ID
+SalesRepID ← SALES_REP
+RouteID ← ROUTEID
+ProductID ← PRODUCT_CODE  (as-is (no letter strip))
+DistributorID ← (literal ???)  (constant "???")
+WarehouseID ← SUPPLIER_ID
+OrderNumber ← ENTRY_ID
+OrderDate ← CHECKINTIME  (dd/MM/yyyy)
+OrderStartTime ← CHECKINTIME  (HH:mm:ss)
+OrderEndTime ← CHECKOUTTIME  (HH:mm:ss)
+OrderStatus ← DELIVERED
+UnitOfMeasure ← PACKAGING
+Currency ← (constant)  (KES)
+QuantityOrdered ← QUANTITY
+AmountOrdered ← TOTAL_VAT_INC
+Discount ← DISCOUNT
+VATAmount ← TOTAL_VAT
+Notes: One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>/api/order</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Order</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>/api/v1/Order</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-order.dwl</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
         </is>
       </c>
     </row>
     <row r="4" ht="220" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>/api/product</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Product</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Product</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-product.dwl</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -863,7 +901,7 @@
 }</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -911,44 +949,62 @@
 }</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="180" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>id ← id
+ProductID ← productcode  (strip leading letters (BIC502418 → 502418))
+product_category ← product_category
+product_name ← product_name
+ProductSKU ← product_desc
+product_status ← product_status
+short_code ← short_code
+tax_code ← tax_code
+hs_code ← hs_code
+focus_product ← focus_product
+tonne_equivalent ← tonne_equivalent
+apply_discount ← apply_discount
+disable_price_check ← disable_price_check
+product_type ← product_type
+supplier ← supplier
+alternative_group ← alternative_group
+supplier_id ← supplier_id
+UnitofMeasure ← uomname
+Notes: productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>/api/product</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Product</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/Product</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-product.dwl</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="220" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>/api/route</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Route</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Route</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-route.dwl</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -992,7 +1048,7 @@
 }</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1016,44 +1072,50 @@
 }</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="180" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>RouteID ← route_id
+RouteName ← route_name
+SalesRepID ← userid
+RouteType ← visit_frequency
+SalesRepType ← saler_category
+Date ← created_at  (dd/MM/yyyy)
+Notes: route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>/api/route</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Route</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>/api/v1/Route</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-route.dwl</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="220" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>SalesRep</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>/api/sales-rep</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_SalesRep</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/SalesRep</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-salesrep.dwl</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1107,7 +1169,7 @@
 }</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1129,44 +1191,49 @@
 }</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="200" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>SalesRepID ← id
+SalesRepName ← name
+DistributorID ← (literal ???)  (constant "???")
+WarehouseID ← warehouse_code
+SalesRepType ← saler_category
+Notes: id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>/api/sales-rep</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>/api/Adapter_SalesRep</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/SalesRep</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-salesrep.dwl</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>/api/customer</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Customer</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Customer</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-customer.dwl</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1268,7 +1335,7 @@
 }</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1308,44 +1375,58 @@
 }</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="180" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>StoreID ← SHOPID
+StoreName ← CUSTOMERNAME
+StoreCategory ← CUSTOMERCATEGORY
+Channel ← CHANNEL
+StoreClassification ← CHANNEL  (same as Channel)
+WarehouseID ← (literal ???)  (constant "???")
+Longitude ← LONGITUDE
+Latitude ← LATITUDE
+City ← LOCATIONNAME
+Region ← REGIONNAME
+County ← (hardcoded empty)  (constant empty)
+StoreStatus ← STATUS
+StoreCreationDate ← DATECREATED  (dd/MM/yyyy)
+StoreSize ← (hardcoded empty)  (constant empty)
+Notes: CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>/api/customer</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Customer</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>/api/v1/Customer</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-customer.dwl</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="220" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>/api/stock</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Stock</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Stock</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-stock.dwl</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1369,7 +1450,7 @@
 }</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1393,44 +1474,50 @@
 }</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="180" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>ProductSKU ← productcode  (from first numeric (BIC969584 → 969584))
+UnitofMeasure ← uomname
+DistributorWarehouseCode ← stockpoint_name
+Date ← date_created  (dd/MM/yyyy)
+InventoryQuantity ← quantity
+InventoryPrice ← total_cost
+Notes: productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>/api/stock</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Stock</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/Stock</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-stock.dwl</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="220" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>/api/warehouse</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>/api/Adapter_Warehouse</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/Warehouse</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>dwl/map-adapter-warehouse.dwl</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>DONE — mapped from real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1532,7 +1619,7 @@
 }</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>{
   "data": [
@@ -1550,9 +1637,1221 @@
 }</t>
         </is>
       </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>WarehouseID ← ID
+WarehouseName ← CUSTOMERNAME
+DistributorID ← (hardcoded empty)  (constant empty)
+Notes: ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>/api/warehouse</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Warehouse</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>/api/v1/Warehouse</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-warehouse.dwl</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SAPI endpoint</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PAPI endpoint</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Exp (EAPI) endpoint</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PAPI mapping file</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Mapping status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SAPI payload</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Transformed payload</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mapping notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>/api/invoice</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Invoice</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Invoice</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-invoice.dwl</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>WAITING for real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>STOREID ← SHOPID
+Discount ← DISCOUNT
+SalesRepID ← USERID
+VATAmount ← TOTAL_VAT
+RouteID ← ROUTEID
+DistributorID ← (property / empty)  (papi.sat.solutech.distributor.id)
+ProductID ← PRODUCT_CODE  (strip leading letters)
+WarehouseID ← SUPPLIER_ID
+OrderNumber ← SALE_ORDER_ID
+InvoiceNumber ← ENTRY_ID
+InvoiceDate ← CREATED_AT  (dd/MM/yyyy)
+InvoiceTime ← CREATED_AT  (HH:mm:ss)
+InvoiceStatus ← PAYMENT_STATUS
+UnitOfMeasure ← PACKAGING
+Currency ← (constant)  (KES)
+QuantityInvoiced ← QUANTITY
+AmountInvoiced ← VALUE_SOLD
+TransType ← ENTRY_TYPE
+Invoice mapping already live. Do not change until you paste SAPI payload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="220" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>/api/order</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Order</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Order</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-order.dwl</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 154,
+      "ENTRY_ID": 60,
+      "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1701,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "FAVOUR SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 89,
+      "PRODUCT_REF": "BIC976044",
+      "PRODUCT_CODE": "BIC976044",
+      "PRODUCT_CATEGORY": "SHAVERS",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
+      "PACKAGING": "PIECE",
+      "QUANTITY": 96,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 22.85,
+      "SELLING_PRICE": 22.67,
+      "VALUE_SOLD": 2176.32,
+      "SALES_VALUE": 1876.137931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T14:03:22",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T14:03:24",
+      "UPDATED_AT": "2026-08-20T14:03:24",
+      "DISCOUNT": 17.28,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 22.67,
+      "PRICE_VAT_EXC": 19.543103,
+      "PRICE_VAT": 3.1268965517,
+      "TOTAL_VAT_INC": 2176.32,
+      "TOTAL_VAT_EXC": 1876.137931,
+      "TOTAL_VAT": 300.1820689655,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T14:02:14",
+      "CHECKOUTTIME": "2026-08-20T14:03:24"
+    },
+    {
+      "ID": 153,
+      "ENTRY_ID": 59,
+      "VISIT_ID": "2e96e08a-19e3-4f6a-ab11-3c9a10d28bdf",
+      "ENTRY_TYPE": "Order",
+      "ERP_REFERENCE": null,
+      "USER_ID": 90,
+      "SALES_REP": "THOMAS OUMA",
+      "REP_CATEGORY": "Van Sales",
+      "SUPERVISOR": "SUPERVISOR",
+      "SHOP_ID": 1704,
+      "CUSTOMER_ERP_CODE": null,
+      "CUSTOMER_NAME": "MOLLYS SHOP",
+      "CUSTOMER_ACCOUNT": null,
+      "USER_CATEGORY": "Van Sales",
+      "CUSTOMER_ADDED_DATE": "2026-08-13T13:56:17",
+      "CUSTOMER_VERIFICATION": "Valid",
+      "CUSTOMER_CATEGORY": "RETAIL SHOP",
+      "LOCATION_ID": 92,
+      "LOCATION_NAME": "LOWER KABETE",
+      "TERRITORY_ID": null,
+      "TERRITORY_NAME": null,
+      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+      "ROUTE_TYPE": "ON",
+      "REGION_NAME": "NAIROBI",
+      "PRODUCT_ID": 8,
+      "PRODUCT_REF": "BIC301209",
+      "PRODUCT_CODE": "BIC301209",
+      "PRODUCT_CATEGORY": "STATIONERY",
+      "PRODUCT_NAME": "BIC",
+      "PRODUCT_SKU": "CRISTAL MED BLU BX 25 LB KE",
+      "PACKAGING": "PACKET",
+      "QUANTITY": 2,
+      "ITEMS_WEIGHT": null,
+      "SALES_VOLUME": null,
+      "BASE_PRICE": 372,
+      "SELLING_PRICE": 372,
+      "VALUE_SOLD": 744,
+      "SALES_VALUE": 641.37931,
+      "CHANNEL": "Physical Visit",
+      "DELIVERED": "Open",
+      "ENTRY_TIME": "2026-08-20T13:38:36",
+      "STAGE_NAME": "New Order",
+      "SUPPLIER_ID": 183,
+      "LPO_NUMBER": null,
+      "PRICELIST_ID": null,
+      "PRICE_LIST": null,
+      "CREATED_AT": "2026-08-20T13:38:38",
+      "UPDATED_AT": "2026-08-20T13:38:38",
+      "DISCOUNT": 0,
+      "VAT_RATE": 16,
+      "PRICE_VAT_INC": 372,
+      "PRICE_VAT_EXC": 320.689655,
+      "PRICE_VAT": 51.3103448276,
+      "TOTAL_VAT_INC": 744,
+      "TOTAL_VAT_EXC": 641.37931,
+      "TOTAL_VAT": 102.6206896552,
+      "ROUTEID": 85,
+      "CHECKINTIME": "2026-08-20T13:37:17",
+      "CHECKOUTTIME": "2026-08-20T13:38:39"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 1701,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC976044",
+      "DistributorID": "???",
+      "WarehouseID": 183,
+      "OrderNumber": 60,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "14:02:14",
+      "OrderEndTime": "14:03:24",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PIECE",
+      "Currency": "KES",
+      "QuantityOrdered": 96,
+      "AmountOrdered": 2176.32,
+      "Discount": 17.28,
+      "VATAmount": 300.1820689655
+    },
+    {
+      "StoreID": 1704,
+      "SalesRepID": "THOMAS OUMA",
+      "RouteID": 85,
+      "ProductID": "BIC301209",
+      "DistributorID": "???",
+      "WarehouseID": 183,
+      "OrderNumber": 59,
+      "OrderDate": "20/08/2026",
+      "OrderStartTime": "13:37:17",
+      "OrderEndTime": "13:38:39",
+      "OrderStatus": "Open",
+      "UnitOfMeasure": "PACKET",
+      "Currency": "KES",
+      "QuantityOrdered": 2,
+      "AmountOrdered": 744,
+      "Discount": 0,
+      "VATAmount": 102.6206896552
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>StoreID ← SHOP_ID
+SalesRepID ← SALES_REP
+RouteID ← ROUTEID
+ProductID ← PRODUCT_CODE  (as-is (no letter strip))
+DistributorID ← (literal ???)  (constant "???")
+WarehouseID ← SUPPLIER_ID
+OrderNumber ← ENTRY_ID
+OrderDate ← CHECKINTIME  (dd/MM/yyyy)
+OrderStartTime ← CHECKINTIME  (HH:mm:ss)
+OrderEndTime ← CHECKOUTTIME  (HH:mm:ss)
+OrderStatus ← DELIVERED
+UnitOfMeasure ← PACKAGING
+Currency ← (constant)  (KES)
+QuantityOrdered ← QUANTITY
+AmountOrdered ← TOTAL_VAT_INC
+Discount ← DISCOUNT
+VATAmount ← TOTAL_VAT
+One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="220" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>/api/product</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Product</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Product</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-product.dwl</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "productcode": "BIC502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    },
+    {
+      "id": 2,
+      "productcode": "BIC502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "product_desc": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "uomname": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 1,
+      "ProductID": "502418",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502418",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    },
+    {
+      "id": 2,
+      "ProductID": "502419",
+      "product_category": "STATIONERY",
+      "product_name": "BIC",
+      "ProductSKU": "CRISTAL MED BLK BX 25 BCL KE",
+      "product_status": "Enabled",
+      "short_code": "BIC502419",
+      "tax_code": "A",
+      "hs_code": null,
+      "focus_product": 0,
+      "tonne_equivalent": null,
+      "apply_discount": null,
+      "disable_price_check": false,
+      "product_type": "item",
+      "supplier": "BIC EAST AFRCA LIMITED",
+      "alternative_group": null,
+      "supplier_id": 2,
+      "UnitofMeasure": "PACKET"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>id ← id
+ProductID ← productcode  (strip leading letters (BIC502418 → 502418))
+product_category ← product_category
+product_name ← product_name
+ProductSKU ← product_desc
+product_status ← product_status
+short_code ← short_code
+tax_code ← tax_code
+hs_code ← hs_code
+focus_product ← focus_product
+tonne_equivalent ← tonne_equivalent
+apply_discount ← apply_discount
+disable_price_check ← disable_price_check
+product_type ← product_type
+supplier ← supplier
+alternative_group ← alternative_group
+supplier_id ← supplier_id
+UnitofMeasure ← uomname
+productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="180" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>/api/route</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Route</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Route</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-route.dwl</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 31,
+      "route_id": 31,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "DICKSON NJUE MONDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:15:47",
+      "updated_at": "2026-06-15T11:15:47",
+      "userid": 75,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "MON",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    },
+    {
+      "id": 33,
+      "route_id": 33,
+      "region_id": 1,
+      "region_name": "NAIROBI",
+      "route_name": "PHILIP DAVID TUESDAY",
+      "routestatus": "Active",
+      "created_by": "CLEMENCEA SARU",
+      "updated_by": null,
+      "created_at": "2026-06-15T11:19:06",
+      "updated_at": "2026-06-15T11:19:06",
+      "userid": 73,
+      "visit_frequency": "Weekly",
+      "visit_week": "1",
+      "visit_day": "TUE",
+      "status": "Active",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "RouteID": 31,
+      "RouteName": "DICKSON NJUE MONDAY",
+      "SalesRepID": 75,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    },
+    {
+      "RouteID": 33,
+      "RouteName": "PHILIP DAVID TUESDAY",
+      "SalesRepID": 73,
+      "RouteType": "Weekly",
+      "SalesRepType": "Van Sales",
+      "Date": "15/06/2026"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>RouteID ← route_id
+RouteName ← route_name
+SalesRepID ← userid
+RouteType ← visit_frequency
+SalesRepType ← saler_category
+Date ← created_at  (dd/MM/yyyy)
+route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SalesRep</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>/api/sales-rep</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_SalesRep</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/SalesRep</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-salesrep.dwl</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "id": 72,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 4,
+      "name": "ESTHER KAGIRI",
+      "email": "ngong@nobleoutlook.co.ke",
+      "phone_number": "0710000000",
+      "last_time_active": "3",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Inactive",
+      "territory_id": null,
+      "rolegroup_id": 4,
+      "vehicle_id": 4,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:40:33",
+      "saler_category": "Drivers (Delivery Agents)"
+    },
+    {
+      "id": 73,
+      "user_reference": null,
+      "warehouse_code": null,
+      "user_type": 2,
+      "user_channel": 1,
+      "region_id": 1,
+      "rep_category": 5,
+      "name": "PHILLIP DAVID",
+      "email": "ngong1@nobleoutlook.co.ke",
+      "phone_number": "0710000001",
+      "last_time_active": "5",
+      "trackactivities": "YES",
+      "demoaccount": "",
+      "billing": "billable",
+      "status": "Active",
+      "territory_id": null,
+      "rolegroup_id": 5,
+      "vehicle_id": 2,
+      "added_by": 3,
+      "created_at": "2026-06-12T06:44:40",
+      "saler_category": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "SalesRepID": 72,
+      "SalesRepName": "ESTHER KAGIRI",
+      "DistributorID": "???",
+      "WarehouseID": "",
+      "SalesRepType": "Drivers (Delivery Agents)"
+    },
+    {
+      "SalesRepID": 73,
+      "SalesRepName": "PHILLIP DAVID",
+      "DistributorID": "???",
+      "WarehouseID": "",
+      "SalesRepType": "Van Sales"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>SalesRepID ← id
+SalesRepName ← name
+DistributorID ← (literal ???)  (constant "???")
+WarehouseID ← warehouse_code
+SalesRepType ← saler_category
+id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="200" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>/api/customer</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Customer</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Customer</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-customer.dwl</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 199,
+      "SHOPID": 199,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "MANDELA SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254722590524",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "IAN MWENDWA",
+      "VERIFIEDDATE": "2026-06-15T14:35:26",
+      "ADDEDBY": "PHILLIP DAVID",
+      "USERID": 73,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "PINCH ANISO",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:27:43",
+      "LASTSALE": "2026-06-15T15:07:50",
+      "LATITUDE": -1.2349905,
+      "LONGITUDE": 36.9328219,
+      "DATECREATED": "2026-06-15T14:17:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    },
+    {
+      "ID": 200,
+      "SHOPID": 200,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 183,
+      "shop_cat_id": 2,
+      "shop_subcat_id": 2,
+      "CUSTOMERCODE": null,
+      "CUSTOMERNAME": "GB SHOP",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 85,
+      "LOCATIONNAME": "RUIRU",
+      "CUSTOMERCATEGORY": "RETAIL SHOP",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "INDIRECT",
+      "SUPPLIER": "GIKAMBURA STOCKPOINT",
+      "PHONENUMBER": "+254725446821",
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "CLEMENCEA SARU",
+      "VERIFIEDDATE": "2026-06-15T16:09:14",
+      "ADDEDBY": "DICKSON NJUE",
+      "USERID": 75,
+      "USERCATEGORY": "Van Sales",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": "GB",
+      "KRAPIN": null,
+      "LASTVISIT": "2026-09-07T15:28:04",
+      "LASTSALE": "2026-08-31T17:08:17",
+      "LATITUDE": -1.2562547,
+      "LONGITUDE": 36.9237899,
+      "DATECREATED": "2026-06-15T16:07:17",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Customer"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "StoreID": 199,
+      "StoreName": "MANDELA SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9328219,
+      "Latitude": -1.2349905,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    },
+    {
+      "StoreID": 200,
+      "StoreName": "GB SHOP",
+      "StoreCategory": "RETAIL SHOP",
+      "Channel": "GENERAL TRADE",
+      "StoreClassification": "GENERAL TRADE",
+      "WarehouseID": "???",
+      "Longitude": 36.9237899,
+      "Latitude": -1.2562547,
+      "City": "RUIRU",
+      "Region": "NAIROBI",
+      "County": "",
+      "StoreStatus": 1,
+      "StoreCreationDate": "15/06/2026",
+      "StoreSize": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>StoreID ← SHOPID
+StoreName ← CUSTOMERNAME
+StoreCategory ← CUSTOMERCATEGORY
+Channel ← CHANNEL
+StoreClassification ← CHANNEL  (same as Channel)
+WarehouseID ← (literal ???)  (constant "???")
+Longitude ← LONGITUDE
+Latitude ← LATITUDE
+City ← LOCATIONNAME
+Region ← REGIONNAME
+County ← (hardcoded empty)  (constant empty)
+StoreStatus ← STATUS
+StoreCreationDate ← DATECREATED  (dd/MM/yyyy)
+StoreSize ← (hardcoded empty)  (constant empty)
+CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="180" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>/api/stock</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Stock</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Stock</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-stock.dwl</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": null,
+      "date_created": "2026-08-17T14:00:56",
+      "quantity": 2640,
+      "total_cost": 1060
+    },
+    {
+      "productcode": "BIC969584",
+      "uomname": "PACKET",
+      "stockpoint_name": "GIKAMBURA STOCKPOINT",
+      "date_created": "2026-08-14T12:42:33",
+      "quantity": 2640,
+      "total_cost": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "",
+      "Date": "17/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1060
+    },
+    {
+      "ProductSKU": "969584",
+      "UnitofMeasure": "PACKET",
+      "DistributorWarehouseCode": "GIKAMBURA STOCKPOINT",
+      "Date": "14/08/2026",
+      "InventoryQuantity": 2640,
+      "InventoryPrice": 1116
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>ProductSKU ← productcode  (from first numeric (BIC969584 → 969584))
+UnitofMeasure ← uomname
+DistributorWarehouseCode ← stockpoint_name
+Date ← date_created  (dd/MM/yyyy)
+InventoryQuantity ← quantity
+InventoryPrice ← total_cost
+productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="180" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>/api/warehouse</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>/api/Adapter_Warehouse</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>/api/v1/Warehouse</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>dwl/map-adapter-warehouse.dwl</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "ID": 183,
+      "SHOPID": 183,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "183",
+      "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 4,
+      "LOCATIONNAME": "GIKAMBURA",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Pending",
+      "VERIFIEDBY": null,
+      "VERIFIEDDATE": null,
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-08T15:07:59",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    },
+    {
+      "ID": 186,
+      "SHOPID": 186,
+      "PARENT_ID": null,
+      "region_id": 1,
+      "group_id": 0,
+      "supplied_by": 0,
+      "shop_cat_id": 1,
+      "shop_subcat_id": null,
+      "CUSTOMERCODE": "186",
+      "CUSTOMERNAME": "NAIROBI WEST STCKPOINT",
+      "IS_HQ": "no",
+      "ACCOUNT_ID": 0,
+      "ACCOUNT": null,
+      "REGIONNAME": "NAIROBI",
+      "LOCATION_ID": 1,
+      "LOCATIONNAME": "NAIROBI WEST",
+      "CUSTOMERCATEGORY": "WHOLESALE",
+      "TERRITORY_NAME": null,
+      "CHANNEL": "GENERAL TRADE",
+      "RELATIONSHIP": "DIRECT",
+      "SUPPLIER": null,
+      "PHONENUMBER": null,
+      "VERIFIED": "Valid",
+      "VERIFIEDBY": "TECLA AYORE",
+      "VERIFIEDDATE": "2026-06-09T22:46:16",
+      "ADDEDBY": "TECLA AYORE",
+      "USERID": 3,
+      "USERCATEGORY": "Admin",
+      "EMAILADDRESS": "",
+      "CONTACTPERSON": null,
+      "KRAPIN": null,
+      "LASTVISIT": null,
+      "LASTSALE": null,
+      "LATITUDE": null,
+      "LONGITUDE": null,
+      "DATECREATED": "2026-06-09T22:42:10",
+      "STATUS": 1,
+      "DISTRIBUTOR_ID": null,
+      "COUNTRY_ID": 113,
+      "COUNTRY_NAME": "KENYA",
+      "CONVERTED_LEAD": "Yes",
+      "CREDIT_LIMIT": 0,
+      "PAYMENT_TERMS": null,
+      "CREDIT_DAYS": null,
+      "CUSTOMER_TYPE": "Supplier"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "data": [
+    {
+      "WarehouseID": 183,
+      "WarehouseName": "GIKAMBURA STOCKPOINT",
+      "DistributorID": ""
+    },
+    {
+      "WarehouseID": 186,
+      "WarehouseName": "NAIROBI WEST STCKPOINT",
+      "DistributorID": ""
+    }
+  ]
+}</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
+          <t>WarehouseID ← ID
+WarehouseName ← CUSTOMERNAME
+DistributorID ← (hardcoded empty)  (constant empty)
+ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +2860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3517,7 +4816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3544,63 +4843,59 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>What I do</t>
+          <t>Where it goes</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Paste one SAPI payload (say which endpoint: Invoice / Order / Product / Route / SalesRep / Customer / Stock / Warehouse)</t>
+          <t>Paste one SAPI payload</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Put the JSON in Endpoints!SAPI payload</t>
+          <t>Payloads!B  (SAPI payload)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Apply / update PAPI Transform Message for that endpoint only</t>
+          <t>PAPI Transform runs; result goes in Payloads!C  (Transformed payload)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Write the mapped JSON into Endpoints!Final payload after PAPI mapping</t>
+          <t>Field-by-field map goes in Payloads!D  (Mapping) and sheet Current field map</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Next SAPI payload</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Push PAPI code and update this Excel</t>
+          <t>Repeat for that resource only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Invoice Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -108,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -132,6 +136,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -560,35 +567,126 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="280" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr"/>
-      <c r="C2" s="7" t="inlineStr"/>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>STOREID ← SHOPID
-Discount ← DISCOUNT
-SalesRepID ← USERID
-VATAmount ← TOTAL_VAT
-RouteID ← ROUTEID
-DistributorID ← (property / empty)  (papi.sat.solutech.distributor.id)
-ProductID ← PRODUCT_CODE  (strip leading letters)
-WarehouseID ← SUPPLIER_ID
-OrderNumber ← SALE_ORDER_ID
-InvoiceNumber ← ENTRY_ID
-InvoiceDate ← CREATED_AT  (dd/MM/yyyy)
-InvoiceTime ← CREATED_AT  (HH:mm:ss)
-InvoiceStatus ← PAYMENT_STATUS
-UnitOfMeasure ← PACKAGING
-Currency ← (constant)  (KES)
-QuantityInvoiced ← QUANTITY
-AmountInvoiced ← VALUE_SOLD
-TransType ← ENTRY_TYPE
-Notes: Invoice mapping already live. Do not change until you paste SAPI payload.</t>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>{
+  "ID": 2227,
+  "ENTRY_ID": 1640,
+  "VISITID": "b4cb0b45-915b-4af6-93b4-fb7b4827f67b",
+  "ENTRY_TYPE": "Sale",
+  "USERID": 75,
+  "SALES_REP": "DICKSON NJUE",
+  "REP_CATEGORY": "Van Sales",
+  "SUPERVISOR": "SUPERVISOR",
+  "SHOPID": 1714,
+  "CUSTOMER_ERP_CODE": null,
+  "CUSTOMER_NAME": "SYNFORMART",
+  "CUSTOMER_ACCOUNT": null,
+  "USERCATEGORY": "Van Sales",
+  "CUSTOMER_ADDED_DATE": "2026-08-13T16:06:24",
+  "CUSTOMER_VERIFICATION": "Valid",
+  "CUSTOMER_CATEGORY": "SHOP AND BROWSER",
+  "LOCATION_ID": 140,
+  "LOCATION_NAME": "Kahawa West",
+  "TERRITORY_ID": null,
+  "TERRITORY_NAME": null,
+  "ROUTE_NAME": "DICKSON NJUE THURSDAY",
+  "ROUTE_TYPE": "ON",
+  "PRODUCT_ID": 87,
+  "REGION_NAME": "NAIROBI",
+  "PRODUCT_REF": "BIC9066113",
+  "PRODUCT_CODE": "BIC9066113",
+  "PRODUCT_CATEGORY": "LIGHTERS",
+  "PRODUCT_NAME": "BIC",
+  "PRODUCT_SKU": "BIC EZ REACH LIGHTER",
+  "PACKAGING_ID": 5,
+  "PACKAGING": "CARD",
+  "ITEMSWEIGHT": null,
+  "SALES_VOLUME": null,
+  "QUANTITY": 1,
+  "BASE_PRICE": 3563.48,
+  "SELLING_PRICE": 3563.48,
+  "VALUE_SOLD": 3563.48,
+  "SALES_VALUE": 3071.9655172413795,
+  "ERP_REFERENCE": null,
+  "DELIVERED": "Delivered",
+  "ENTRY_TIME": "2026-08-13T16:11:19",
+  "TAX_INVOICE_NO": "0111778770000014123",
+  "CU_SERIAL_NO": "KRAMW011202209177877",
+  "SALE_ORDER_ID": null,
+  "STAGE_NAME": null,
+  "SUPPLIER_ID": 0,
+  "CHANNEL": "Physical Visit",
+  "PAYMENT_METHOD": "cash",
+  "PAYMENT_STATUS": "Fully Paid",
+  "AMOUNT_PAID": 6773.59,
+  "LPO_NUMBER": null,
+  "PRICELIST_ID": null,
+  "PRICE_LIST": null,
+  "CREATED_AT": "2026-08-13T16:11:25",
+  "UPDATED_AT": "2026-08-13T16:11:25",
+  "DISCOUNT": 0,
+  "VAT_RATE": 16,
+  "PRICE_VAT_INC": 3563.48,
+  "PRICE_VAT_EXC": 3071.965517,
+  "PRICE_VAT": 491.5144827586,
+  "TOTAL_VAT_INC": 3563.48,
+  "TOTAL_VAT_EXC": 3071.965517,
+  "TOTAL_VAT": 491.5144827586,
+  "ROUTEID": 42
+}</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>{
+  "STOREID": 1714,
+  "Discount": 0,
+  "SalesRepID": 75,
+  "VATAmount": 491.5144827586,
+  "RouteID": 42,
+  "DistributorID": "",
+  "ProductID": "9066113",
+  "WarehouseID": 0,
+  "OrderNumber": "",
+  "InvoiceNumber": 1640,
+  "InvoiceDate": "13/08/2026",
+  "InvoiceTime": "16:11:25",
+  "InvoiceStatus": "Fully Paid",
+  "UnitOfMeasure": "CARD",
+  "Currency": "KES",
+  "QuantityInvoiced": 1,
+  "AmountInvoiced": 3563.48,
+  "TransType": "Sale"
+}</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>SHOPID -&gt; STOREID
+DISCOUNT -&gt; Discount
+USERID -&gt; SalesRepID
+TOTAL_VAT -&gt; VATAmount
+ROUTEID -&gt; RouteID
+'' -&gt; DistributorID
+PRODUCT_CODE -&gt; ProductID
+SUPPLIER_ID -&gt; WarehouseID
+SALE_ORDER_ID -&gt; OrderNumber
+ENTRY_ID -&gt; InvoiceNumber
+CREATED_AT -&gt; InvoiceDate
+CREATED_AT -&gt; InvoiceTime
+PAYMENT_STATUS -&gt; InvoiceStatus
+PACKAGING -&gt; UnitOfMeasure
+'' -&gt; Currency
+QUANTITY -&gt; QuantityInvoiced
+VALUE_SOLD -&gt; AmountInvoiced
+ENTRY_TYPE -&gt; TransType</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -613,7 +711,7 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>WAITING for real SAPI payload</t>
+          <t>DONE — mapped from real SAPI payload</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1842,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="280" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Invoice</t>
@@ -1772,32 +1870,123 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>WAITING for real SAPI payload</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>DONE — mapped from real SAPI payload</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "ID": 2227,
+  "ENTRY_ID": 1640,
+  "VISITID": "b4cb0b45-915b-4af6-93b4-fb7b4827f67b",
+  "ENTRY_TYPE": "Sale",
+  "USERID": 75,
+  "SALES_REP": "DICKSON NJUE",
+  "REP_CATEGORY": "Van Sales",
+  "SUPERVISOR": "SUPERVISOR",
+  "SHOPID": 1714,
+  "CUSTOMER_ERP_CODE": null,
+  "CUSTOMER_NAME": "SYNFORMART",
+  "CUSTOMER_ACCOUNT": null,
+  "USERCATEGORY": "Van Sales",
+  "CUSTOMER_ADDED_DATE": "2026-08-13T16:06:24",
+  "CUSTOMER_VERIFICATION": "Valid",
+  "CUSTOMER_CATEGORY": "SHOP AND BROWSER",
+  "LOCATION_ID": 140,
+  "LOCATION_NAME": "Kahawa West",
+  "TERRITORY_ID": null,
+  "TERRITORY_NAME": null,
+  "ROUTE_NAME": "DICKSON NJUE THURSDAY",
+  "ROUTE_TYPE": "ON",
+  "PRODUCT_ID": 87,
+  "REGION_NAME": "NAIROBI",
+  "PRODUCT_REF": "BIC9066113",
+  "PRODUCT_CODE": "BIC9066113",
+  "PRODUCT_CATEGORY": "LIGHTERS",
+  "PRODUCT_NAME": "BIC",
+  "PRODUCT_SKU": "BIC EZ REACH LIGHTER",
+  "PACKAGING_ID": 5,
+  "PACKAGING": "CARD",
+  "ITEMSWEIGHT": null,
+  "SALES_VOLUME": null,
+  "QUANTITY": 1,
+  "BASE_PRICE": 3563.48,
+  "SELLING_PRICE": 3563.48,
+  "VALUE_SOLD": 3563.48,
+  "SALES_VALUE": 3071.9655172413795,
+  "ERP_REFERENCE": null,
+  "DELIVERED": "Delivered",
+  "ENTRY_TIME": "2026-08-13T16:11:19",
+  "TAX_INVOICE_NO": "0111778770000014123",
+  "CU_SERIAL_NO": "KRAMW011202209177877",
+  "SALE_ORDER_ID": null,
+  "STAGE_NAME": null,
+  "SUPPLIER_ID": 0,
+  "CHANNEL": "Physical Visit",
+  "PAYMENT_METHOD": "cash",
+  "PAYMENT_STATUS": "Fully Paid",
+  "AMOUNT_PAID": 6773.59,
+  "LPO_NUMBER": null,
+  "PRICELIST_ID": null,
+  "PRICE_LIST": null,
+  "CREATED_AT": "2026-08-13T16:11:25",
+  "UPDATED_AT": "2026-08-13T16:11:25",
+  "DISCOUNT": 0,
+  "VAT_RATE": 16,
+  "PRICE_VAT_INC": 3563.48,
+  "PRICE_VAT_EXC": 3071.965517,
+  "PRICE_VAT": 491.5144827586,
+  "TOTAL_VAT_INC": 3563.48,
+  "TOTAL_VAT_EXC": 3071.965517,
+  "TOTAL_VAT": 491.5144827586,
+  "ROUTEID": 42
+}</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "STOREID": 1714,
+  "Discount": 0,
+  "SalesRepID": 75,
+  "VATAmount": 491.5144827586,
+  "RouteID": 42,
+  "DistributorID": "",
+  "ProductID": "9066113",
+  "WarehouseID": 0,
+  "OrderNumber": "",
+  "InvoiceNumber": 1640,
+  "InvoiceDate": "13/08/2026",
+  "InvoiceTime": "16:11:25",
+  "InvoiceStatus": "Fully Paid",
+  "UnitOfMeasure": "CARD",
+  "Currency": "KES",
+  "QuantityInvoiced": 1,
+  "AmountInvoiced": 3563.48,
+  "TransType": "Sale"
+}</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>STOREID ← SHOPID
-Discount ← DISCOUNT
-SalesRepID ← USERID
-VATAmount ← TOTAL_VAT
-RouteID ← ROUTEID
-DistributorID ← (property / empty)  (papi.sat.solutech.distributor.id)
-ProductID ← PRODUCT_CODE  (strip leading letters)
-WarehouseID ← SUPPLIER_ID
-OrderNumber ← SALE_ORDER_ID
-InvoiceNumber ← ENTRY_ID
-InvoiceDate ← CREATED_AT  (dd/MM/yyyy)
-InvoiceTime ← CREATED_AT  (HH:mm:ss)
-InvoiceStatus ← PAYMENT_STATUS
-UnitOfMeasure ← PACKAGING
-Currency ← (constant)  (KES)
-QuantityInvoiced ← QUANTITY
-AmountInvoiced ← VALUE_SOLD
-TransType ← ENTRY_TYPE
-Invoice mapping already live. Do not change until you paste SAPI payload.</t>
+          <t>SHOPID -&gt; STOREID
+DISCOUNT -&gt; Discount
+USERID -&gt; SalesRepID
+TOTAL_VAT -&gt; VATAmount
+ROUTEID -&gt; RouteID
+'' -&gt; DistributorID
+PRODUCT_CODE -&gt; ProductID
+SUPPLIER_ID -&gt; WarehouseID
+SALE_ORDER_ID -&gt; OrderNumber
+ENTRY_ID -&gt; InvoiceNumber
+CREATED_AT -&gt; InvoiceDate
+CREATED_AT -&gt; InvoiceTime
+PAYMENT_STATUS -&gt; InvoiceStatus
+PACKAGING -&gt; UnitOfMeasure
+'' -&gt; Currency
+QUANTITY -&gt; QuantityInvoiced
+VALUE_SOLD -&gt; AmountInvoiced
+ENTRY_TYPE -&gt; TransType</t>
         </is>
       </c>
     </row>
@@ -2915,7 +3104,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SHOPID -&gt; STOREID</t>
         </is>
       </c>
     </row>
@@ -2937,7 +3126,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>DISCOUNT -&gt; Discount</t>
         </is>
       </c>
     </row>
@@ -2959,7 +3148,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>USERID -&gt; SalesRepID</t>
         </is>
       </c>
     </row>
@@ -2981,7 +3170,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3192,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ROUTEID -&gt; RouteID</t>
         </is>
       </c>
     </row>
@@ -3020,12 +3209,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>(property / empty)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>papi.sat.solutech.distributor.id</t>
+          <t>'' -&gt; DistributorID</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3236,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters</t>
+          <t>PRODUCT_CODE -&gt; ProductID</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3258,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SUPPLIER_ID -&gt; WarehouseID</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3280,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SALE_ORDER_ID -&gt; OrderNumber</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3302,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ENTRY_ID -&gt; InvoiceNumber</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3324,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>CREATED_AT -&gt; InvoiceDate</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3346,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>HH:mm:ss</t>
+          <t>CREATED_AT -&gt; InvoiceTime</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3368,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>PAYMENT_STATUS -&gt; InvoiceStatus</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3390,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>PACKAGING -&gt; UnitOfMeasure</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3407,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>(constant)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>KES</t>
+          <t>'' -&gt; Currency</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3434,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>QUANTITY -&gt; QuantityInvoiced</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3456,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>VALUE_SOLD -&gt; AmountInvoiced</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3478,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ENTRY_TYPE -&gt; TransType</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Order Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -139,6 +139,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -715,208 +718,119 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="220" customHeight="1">
+    <row r="3" ht="280" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 154,
-      "ENTRY_ID": 60,
-      "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
-      "ENTRY_TYPE": "Order",
-      "ERP_REFERENCE": null,
-      "USER_ID": 90,
-      "SALES_REP": "THOMAS OUMA",
-      "REP_CATEGORY": "Van Sales",
-      "SUPERVISOR": "SUPERVISOR",
-      "SHOP_ID": 1701,
-      "CUSTOMER_ERP_CODE": null,
-      "CUSTOMER_NAME": "FAVOUR SHOP",
-      "CUSTOMER_ACCOUNT": null,
-      "USER_CATEGORY": "Van Sales",
-      "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
-      "CUSTOMER_VERIFICATION": "Valid",
-      "CUSTOMER_CATEGORY": "RETAIL SHOP",
-      "LOCATION_ID": 92,
-      "LOCATION_NAME": "LOWER KABETE",
-      "TERRITORY_ID": null,
-      "TERRITORY_NAME": null,
-      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
-      "ROUTE_TYPE": "ON",
-      "REGION_NAME": "NAIROBI",
-      "PRODUCT_ID": 89,
-      "PRODUCT_REF": "BIC976044",
-      "PRODUCT_CODE": "BIC976044",
-      "PRODUCT_CATEGORY": "SHAVERS",
-      "PRODUCT_NAME": "BIC",
-      "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
-      "PACKAGING": "PIECE",
-      "QUANTITY": 96,
-      "ITEMS_WEIGHT": null,
-      "SALES_VOLUME": null,
-      "BASE_PRICE": 22.85,
-      "SELLING_PRICE": 22.67,
-      "VALUE_SOLD": 2176.32,
-      "SALES_VALUE": 1876.137931,
-      "CHANNEL": "Physical Visit",
-      "DELIVERED": "Open",
-      "ENTRY_TIME": "2026-08-20T14:03:22",
-      "STAGE_NAME": "New Order",
-      "SUPPLIER_ID": 183,
-      "LPO_NUMBER": null,
-      "PRICELIST_ID": null,
-      "PRICE_LIST": null,
-      "CREATED_AT": "2026-08-20T14:03:24",
-      "UPDATED_AT": "2026-08-20T14:03:24",
-      "DISCOUNT": 17.28,
-      "VAT_RATE": 16,
-      "PRICE_VAT_INC": 22.67,
-      "PRICE_VAT_EXC": 19.543103,
-      "PRICE_VAT": 3.1268965517,
-      "TOTAL_VAT_INC": 2176.32,
-      "TOTAL_VAT_EXC": 1876.137931,
-      "TOTAL_VAT": 300.1820689655,
-      "ROUTEID": 85,
-      "CHECKINTIME": "2026-08-20T14:02:14",
-      "CHECKOUTTIME": "2026-08-20T14:03:24"
-    },
-    {
-      "ID": 153,
-      "ENTRY_ID": 59,
-      "VISIT_ID": "2e96e08a-19e3-4f6a-ab11-3c9a10d28bdf",
-      "ENTRY_TYPE": "Order",
-      "ERP_REFERENCE": null,
-      "USER_ID": 90,
-      "SALES_REP": "THOMAS OUMA",
-      "REP_CATEGORY": "Van Sales",
-      "SUPERVISOR": "SUPERVISOR",
-      "SHOP_ID": 1704,
-      "CUSTOMER_ERP_CODE": null,
-      "CUSTOMER_NAME": "MOLLYS SHOP",
-      "CUSTOMER_ACCOUNT": null,
-      "USER_CATEGORY": "Van Sales",
-      "CUSTOMER_ADDED_DATE": "2026-08-13T13:56:17",
-      "CUSTOMER_VERIFICATION": "Valid",
-      "CUSTOMER_CATEGORY": "RETAIL SHOP",
-      "LOCATION_ID": 92,
-      "LOCATION_NAME": "LOWER KABETE",
-      "TERRITORY_ID": null,
-      "TERRITORY_NAME": null,
-      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
-      "ROUTE_TYPE": "ON",
-      "REGION_NAME": "NAIROBI",
-      "PRODUCT_ID": 8,
-      "PRODUCT_REF": "BIC301209",
-      "PRODUCT_CODE": "BIC301209",
-      "PRODUCT_CATEGORY": "STATIONERY",
-      "PRODUCT_NAME": "BIC",
-      "PRODUCT_SKU": "CRISTAL MED BLU BX 25 LB KE",
-      "PACKAGING": "PACKET",
-      "QUANTITY": 2,
-      "ITEMS_WEIGHT": null,
-      "SALES_VOLUME": null,
-      "BASE_PRICE": 372,
-      "SELLING_PRICE": 372,
-      "VALUE_SOLD": 744,
-      "SALES_VALUE": 641.37931,
-      "CHANNEL": "Physical Visit",
-      "DELIVERED": "Open",
-      "ENTRY_TIME": "2026-08-20T13:38:36",
-      "STAGE_NAME": "New Order",
-      "SUPPLIER_ID": 183,
-      "LPO_NUMBER": null,
-      "PRICELIST_ID": null,
-      "PRICE_LIST": null,
-      "CREATED_AT": "2026-08-20T13:38:38",
-      "UPDATED_AT": "2026-08-20T13:38:38",
-      "DISCOUNT": 0,
-      "VAT_RATE": 16,
-      "PRICE_VAT_INC": 372,
-      "PRICE_VAT_EXC": 320.689655,
-      "PRICE_VAT": 51.3103448276,
-      "TOTAL_VAT_INC": 744,
-      "TOTAL_VAT_EXC": 641.37931,
-      "TOTAL_VAT": 102.6206896552,
-      "ROUTEID": 85,
-      "CHECKINTIME": "2026-08-20T13:37:17",
-      "CHECKOUTTIME": "2026-08-20T13:38:39"
-    }
-  ]
+  "ID": 154,
+  "ENTRY_ID": 60,
+  "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
+  "ENTRY_TYPE": "Order",
+  "ERP_REFERENCE": null,
+  "USER_ID": 90,
+  "SALES_REP": "THOMAS OUMA",
+  "REP_CATEGORY": "Van Sales",
+  "SUPERVISOR": "SUPERVISOR",
+  "SHOP_ID": 1701,
+  "CUSTOMER_ERP_CODE": null,
+  "CUSTOMER_NAME": "FAVOUR SHOP",
+  "CUSTOMER_ACCOUNT": null,
+  "USER_CATEGORY": "Van Sales",
+  "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
+  "CUSTOMER_VERIFICATION": "Valid",
+  "CUSTOMER_CATEGORY": "RETAIL SHOP",
+  "LOCATION_ID": 92,
+  "LOCATION_NAME": "LOWER KABETE",
+  "TERRITORY_ID": null,
+  "TERRITORY_NAME": null,
+  "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+  "ROUTE_TYPE": "ON",
+  "REGION_NAME": "NAIROBI",
+  "PRODUCT_ID": 89,
+  "PRODUCT_REF": "BIC976044",
+  "PRODUCT_CODE": "BIC976044",
+  "PRODUCT_CATEGORY": "SHAVERS",
+  "PRODUCT_NAME": "BIC",
+  "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
+  "PACKAGING": "PIECE",
+  "QUANTITY": 96,
+  "ITEMS_WEIGHT": null,
+  "SALES_VOLUME": null,
+  "BASE_PRICE": 22.85,
+  "SELLING_PRICE": 22.67,
+  "VALUE_SOLD": 2176.32,
+  "SALES_VALUE": 1876.137931,
+  "CHANNEL": "Physical Visit",
+  "DELIVERED": "Open",
+  "ENTRY_TIME": "2026-08-20T14:03:22",
+  "STAGE_NAME": "New Order",
+  "SUPPLIER_ID": 183,
+  "LPO_NUMBER": null,
+  "PRICELIST_ID": null,
+  "PRICE_LIST": null,
+  "CREATED_AT": "2026-08-20T14:03:24",
+  "UPDATED_AT": "2026-08-20T14:03:24",
+  "DISCOUNT": 17.28,
+  "VAT_RATE": 16,
+  "PRICE_VAT_INC": 22.67,
+  "PRICE_VAT_EXC": 19.543103,
+  "PRICE_VAT": 3.1268965517,
+  "TOTAL_VAT_INC": 2176.32,
+  "TOTAL_VAT_EXC": 1876.137931,
+  "TOTAL_VAT": 300.1820689655,
+  "ROUTEID": 85,
+  "CHECKINTIME": "2026-08-20T14:02:14",
+  "CHECKOUTTIME": "2026-08-20T14:03:24"
 }</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "StoreID": 1701,
-      "SalesRepID": "THOMAS OUMA",
-      "RouteID": 85,
-      "ProductID": "BIC976044",
-      "DistributorID": "???",
-      "WarehouseID": 183,
-      "OrderNumber": 60,
-      "OrderDate": "20/08/2026",
-      "OrderStartTime": "14:02:14",
-      "OrderEndTime": "14:03:24",
-      "OrderStatus": "Open",
-      "UnitOfMeasure": "PIECE",
-      "Currency": "KES",
-      "QuantityOrdered": 96,
-      "AmountOrdered": 2176.32,
-      "Discount": 17.28,
-      "VATAmount": 300.1820689655
-    },
-    {
-      "StoreID": 1704,
-      "SalesRepID": "THOMAS OUMA",
-      "RouteID": 85,
-      "ProductID": "BIC301209",
-      "DistributorID": "???",
-      "WarehouseID": 183,
-      "OrderNumber": 59,
-      "OrderDate": "20/08/2026",
-      "OrderStartTime": "13:37:17",
-      "OrderEndTime": "13:38:39",
-      "OrderStatus": "Open",
-      "UnitOfMeasure": "PACKET",
-      "Currency": "KES",
-      "QuantityOrdered": 2,
-      "AmountOrdered": 744,
-      "Discount": 0,
-      "VATAmount": 102.6206896552
-    }
-  ]
+  "StoreID": 1701,
+  "SalesRepID": "THOMAS OUMA",
+  "RouteID": 85,
+  "ProductID": "BIC976044",
+  "DistributorID": "???",
+  "WarehouseID": 183,
+  "OrderNumber": 60,
+  "OrderDate": "20/08/2026",
+  "OrderStartTime": "14:02:14",
+  "OrderEndTime": "14:03:24",
+  "OrderStatus": "Open",
+  "UnitOfMeasure": "PIECE",
+  "Currency": "KES",
+  "QuantityOrdered": 96,
+  "AmountOrdered": 2176.32,
+  "Discount": 17.28,
+  "VATAmount": 300.1820689655
 }</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>StoreID ← SHOP_ID
-SalesRepID ← SALES_REP
-RouteID ← ROUTEID
-ProductID ← PRODUCT_CODE  (as-is (no letter strip))
-DistributorID ← (literal ???)  (constant "???")
-WarehouseID ← SUPPLIER_ID
-OrderNumber ← ENTRY_ID
-OrderDate ← CHECKINTIME  (dd/MM/yyyy)
-OrderStartTime ← CHECKINTIME  (HH:mm:ss)
-OrderEndTime ← CHECKOUTTIME  (HH:mm:ss)
-OrderStatus ← DELIVERED
-UnitOfMeasure ← PACKAGING
-Currency ← (constant)  (KES)
-QuantityOrdered ← QUANTITY
-AmountOrdered ← TOTAL_VAT_INC
-Discount ← DISCOUNT
-VATAmount ← TOTAL_VAT
-Notes: One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>SHOP_ID -&gt; StoreID
+SALES_REP -&gt; SalesRepID
+ROUTEID -&gt; RouteID
+PRODUCT_CODE -&gt; ProductID
+'' -&gt; DistributorID
+SUPPLIER_ID -&gt; WarehouseID
+ENTRY_ID -&gt; OrderNumber
+CHECKINTIME -&gt; OrderDate
+CHECKINTIME -&gt; OrderStartTime
+CHECKOUTTIME -&gt; OrderEndTime
+DELIVERED -&gt; OrderStatus
+PACKAGING -&gt; UnitOfMeasure
+'' -&gt; Currency
+QUANTITY -&gt; QuantityOrdered
+TOTAL_VAT_INC -&gt; AmountOrdered
+DISCOUNT -&gt; Discount
+TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -1990,7 +1904,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="220" customHeight="1">
+    <row r="3" ht="280" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Order</t>
@@ -2024,199 +1938,110 @@
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 154,
-      "ENTRY_ID": 60,
-      "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
-      "ENTRY_TYPE": "Order",
-      "ERP_REFERENCE": null,
-      "USER_ID": 90,
-      "SALES_REP": "THOMAS OUMA",
-      "REP_CATEGORY": "Van Sales",
-      "SUPERVISOR": "SUPERVISOR",
-      "SHOP_ID": 1701,
-      "CUSTOMER_ERP_CODE": null,
-      "CUSTOMER_NAME": "FAVOUR SHOP",
-      "CUSTOMER_ACCOUNT": null,
-      "USER_CATEGORY": "Van Sales",
-      "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
-      "CUSTOMER_VERIFICATION": "Valid",
-      "CUSTOMER_CATEGORY": "RETAIL SHOP",
-      "LOCATION_ID": 92,
-      "LOCATION_NAME": "LOWER KABETE",
-      "TERRITORY_ID": null,
-      "TERRITORY_NAME": null,
-      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
-      "ROUTE_TYPE": "ON",
-      "REGION_NAME": "NAIROBI",
-      "PRODUCT_ID": 89,
-      "PRODUCT_REF": "BIC976044",
-      "PRODUCT_CODE": "BIC976044",
-      "PRODUCT_CATEGORY": "SHAVERS",
-      "PRODUCT_NAME": "BIC",
-      "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
-      "PACKAGING": "PIECE",
-      "QUANTITY": 96,
-      "ITEMS_WEIGHT": null,
-      "SALES_VOLUME": null,
-      "BASE_PRICE": 22.85,
-      "SELLING_PRICE": 22.67,
-      "VALUE_SOLD": 2176.32,
-      "SALES_VALUE": 1876.137931,
-      "CHANNEL": "Physical Visit",
-      "DELIVERED": "Open",
-      "ENTRY_TIME": "2026-08-20T14:03:22",
-      "STAGE_NAME": "New Order",
-      "SUPPLIER_ID": 183,
-      "LPO_NUMBER": null,
-      "PRICELIST_ID": null,
-      "PRICE_LIST": null,
-      "CREATED_AT": "2026-08-20T14:03:24",
-      "UPDATED_AT": "2026-08-20T14:03:24",
-      "DISCOUNT": 17.28,
-      "VAT_RATE": 16,
-      "PRICE_VAT_INC": 22.67,
-      "PRICE_VAT_EXC": 19.543103,
-      "PRICE_VAT": 3.1268965517,
-      "TOTAL_VAT_INC": 2176.32,
-      "TOTAL_VAT_EXC": 1876.137931,
-      "TOTAL_VAT": 300.1820689655,
-      "ROUTEID": 85,
-      "CHECKINTIME": "2026-08-20T14:02:14",
-      "CHECKOUTTIME": "2026-08-20T14:03:24"
-    },
-    {
-      "ID": 153,
-      "ENTRY_ID": 59,
-      "VISIT_ID": "2e96e08a-19e3-4f6a-ab11-3c9a10d28bdf",
-      "ENTRY_TYPE": "Order",
-      "ERP_REFERENCE": null,
-      "USER_ID": 90,
-      "SALES_REP": "THOMAS OUMA",
-      "REP_CATEGORY": "Van Sales",
-      "SUPERVISOR": "SUPERVISOR",
-      "SHOP_ID": 1704,
-      "CUSTOMER_ERP_CODE": null,
-      "CUSTOMER_NAME": "MOLLYS SHOP",
-      "CUSTOMER_ACCOUNT": null,
-      "USER_CATEGORY": "Van Sales",
-      "CUSTOMER_ADDED_DATE": "2026-08-13T13:56:17",
-      "CUSTOMER_VERIFICATION": "Valid",
-      "CUSTOMER_CATEGORY": "RETAIL SHOP",
-      "LOCATION_ID": 92,
-      "LOCATION_NAME": "LOWER KABETE",
-      "TERRITORY_ID": null,
-      "TERRITORY_NAME": null,
-      "ROUTE_NAME": "THOMAS OUMA THURSDAY",
-      "ROUTE_TYPE": "ON",
-      "REGION_NAME": "NAIROBI",
-      "PRODUCT_ID": 8,
-      "PRODUCT_REF": "BIC301209",
-      "PRODUCT_CODE": "BIC301209",
-      "PRODUCT_CATEGORY": "STATIONERY",
-      "PRODUCT_NAME": "BIC",
-      "PRODUCT_SKU": "CRISTAL MED BLU BX 25 LB KE",
-      "PACKAGING": "PACKET",
-      "QUANTITY": 2,
-      "ITEMS_WEIGHT": null,
-      "SALES_VOLUME": null,
-      "BASE_PRICE": 372,
-      "SELLING_PRICE": 372,
-      "VALUE_SOLD": 744,
-      "SALES_VALUE": 641.37931,
-      "CHANNEL": "Physical Visit",
-      "DELIVERED": "Open",
-      "ENTRY_TIME": "2026-08-20T13:38:36",
-      "STAGE_NAME": "New Order",
-      "SUPPLIER_ID": 183,
-      "LPO_NUMBER": null,
-      "PRICELIST_ID": null,
-      "PRICE_LIST": null,
-      "CREATED_AT": "2026-08-20T13:38:38",
-      "UPDATED_AT": "2026-08-20T13:38:38",
-      "DISCOUNT": 0,
-      "VAT_RATE": 16,
-      "PRICE_VAT_INC": 372,
-      "PRICE_VAT_EXC": 320.689655,
-      "PRICE_VAT": 51.3103448276,
-      "TOTAL_VAT_INC": 744,
-      "TOTAL_VAT_EXC": 641.37931,
-      "TOTAL_VAT": 102.6206896552,
-      "ROUTEID": 85,
-      "CHECKINTIME": "2026-08-20T13:37:17",
-      "CHECKOUTTIME": "2026-08-20T13:38:39"
-    }
-  ]
+  "ID": 154,
+  "ENTRY_ID": 60,
+  "VISIT_ID": "1bca9799-849e-488d-8517-662468133a6f",
+  "ENTRY_TYPE": "Order",
+  "ERP_REFERENCE": null,
+  "USER_ID": 90,
+  "SALES_REP": "THOMAS OUMA",
+  "REP_CATEGORY": "Van Sales",
+  "SUPERVISOR": "SUPERVISOR",
+  "SHOP_ID": 1701,
+  "CUSTOMER_ERP_CODE": null,
+  "CUSTOMER_NAME": "FAVOUR SHOP",
+  "CUSTOMER_ACCOUNT": null,
+  "USER_CATEGORY": "Van Sales",
+  "CUSTOMER_ADDED_DATE": "2026-08-13T13:25:30",
+  "CUSTOMER_VERIFICATION": "Valid",
+  "CUSTOMER_CATEGORY": "RETAIL SHOP",
+  "LOCATION_ID": 92,
+  "LOCATION_NAME": "LOWER KABETE",
+  "TERRITORY_ID": null,
+  "TERRITORY_NAME": null,
+  "ROUTE_NAME": "THOMAS OUMA THURSDAY",
+  "ROUTE_TYPE": "ON",
+  "REGION_NAME": "NAIROBI",
+  "PRODUCT_ID": 89,
+  "PRODUCT_REF": "BIC976044",
+  "PRODUCT_CODE": "BIC976044",
+  "PRODUCT_CATEGORY": "SHAVERS",
+  "PRODUCT_NAME": "BIC",
+  "PRODUCT_SKU": "BIC 1 RAZOR SINGLE POUCH",
+  "PACKAGING": "PIECE",
+  "QUANTITY": 96,
+  "ITEMS_WEIGHT": null,
+  "SALES_VOLUME": null,
+  "BASE_PRICE": 22.85,
+  "SELLING_PRICE": 22.67,
+  "VALUE_SOLD": 2176.32,
+  "SALES_VALUE": 1876.137931,
+  "CHANNEL": "Physical Visit",
+  "DELIVERED": "Open",
+  "ENTRY_TIME": "2026-08-20T14:03:22",
+  "STAGE_NAME": "New Order",
+  "SUPPLIER_ID": 183,
+  "LPO_NUMBER": null,
+  "PRICELIST_ID": null,
+  "PRICE_LIST": null,
+  "CREATED_AT": "2026-08-20T14:03:24",
+  "UPDATED_AT": "2026-08-20T14:03:24",
+  "DISCOUNT": 17.28,
+  "VAT_RATE": 16,
+  "PRICE_VAT_INC": 22.67,
+  "PRICE_VAT_EXC": 19.543103,
+  "PRICE_VAT": 3.1268965517,
+  "TOTAL_VAT_INC": 2176.32,
+  "TOTAL_VAT_EXC": 1876.137931,
+  "TOTAL_VAT": 300.1820689655,
+  "ROUTEID": 85,
+  "CHECKINTIME": "2026-08-20T14:02:14",
+  "CHECKOUTTIME": "2026-08-20T14:03:24"
 }</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "StoreID": 1701,
-      "SalesRepID": "THOMAS OUMA",
-      "RouteID": 85,
-      "ProductID": "BIC976044",
-      "DistributorID": "???",
-      "WarehouseID": 183,
-      "OrderNumber": 60,
-      "OrderDate": "20/08/2026",
-      "OrderStartTime": "14:02:14",
-      "OrderEndTime": "14:03:24",
-      "OrderStatus": "Open",
-      "UnitOfMeasure": "PIECE",
-      "Currency": "KES",
-      "QuantityOrdered": 96,
-      "AmountOrdered": 2176.32,
-      "Discount": 17.28,
-      "VATAmount": 300.1820689655
-    },
-    {
-      "StoreID": 1704,
-      "SalesRepID": "THOMAS OUMA",
-      "RouteID": 85,
-      "ProductID": "BIC301209",
-      "DistributorID": "???",
-      "WarehouseID": 183,
-      "OrderNumber": 59,
-      "OrderDate": "20/08/2026",
-      "OrderStartTime": "13:37:17",
-      "OrderEndTime": "13:38:39",
-      "OrderStatus": "Open",
-      "UnitOfMeasure": "PACKET",
-      "Currency": "KES",
-      "QuantityOrdered": 2,
-      "AmountOrdered": 744,
-      "Discount": 0,
-      "VATAmount": 102.6206896552
-    }
-  ]
+  "StoreID": 1701,
+  "SalesRepID": "THOMAS OUMA",
+  "RouteID": 85,
+  "ProductID": "BIC976044",
+  "DistributorID": "???",
+  "WarehouseID": 183,
+  "OrderNumber": 60,
+  "OrderDate": "20/08/2026",
+  "OrderStartTime": "14:02:14",
+  "OrderEndTime": "14:03:24",
+  "OrderStatus": "Open",
+  "UnitOfMeasure": "PIECE",
+  "Currency": "KES",
+  "QuantityOrdered": 96,
+  "AmountOrdered": 2176.32,
+  "Discount": 17.28,
+  "VATAmount": 300.1820689655
 }</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>StoreID ← SHOP_ID
-SalesRepID ← SALES_REP
-RouteID ← ROUTEID
-ProductID ← PRODUCT_CODE  (as-is (no letter strip))
-DistributorID ← (literal ???)  (constant "???")
-WarehouseID ← SUPPLIER_ID
-OrderNumber ← ENTRY_ID
-OrderDate ← CHECKINTIME  (dd/MM/yyyy)
-OrderStartTime ← CHECKINTIME  (HH:mm:ss)
-OrderEndTime ← CHECKOUTTIME  (HH:mm:ss)
-OrderStatus ← DELIVERED
-UnitOfMeasure ← PACKAGING
-Currency ← (constant)  (KES)
-QuantityOrdered ← QUANTITY
-AmountOrdered ← TOTAL_VAT_INC
-Discount ← DISCOUNT
-VATAmount ← TOTAL_VAT
-One SAPI field per PAPI field. SHOP_ID, SALES_REP, ROUTEID, PRODUCT_CODE, SUPPLIER_ID, ENTRY_ID, CHECKINTIME, CHECKOUTTIME, DELIVERED, PACKAGING, QUANTITY, TOTAL_VAT_INC, DISCOUNT, TOTAL_VAT. DistributorID is ???. Currency KES. Dates dd/MM/yyyy and HH:mm:ss. ProductID is PRODUCT_CODE as returned (no letter strip).</t>
+          <t>SHOP_ID -&gt; StoreID
+SALES_REP -&gt; SalesRepID
+ROUTEID -&gt; RouteID
+PRODUCT_CODE -&gt; ProductID
+'' -&gt; DistributorID
+SUPPLIER_ID -&gt; WarehouseID
+ENTRY_ID -&gt; OrderNumber
+CHECKINTIME -&gt; OrderDate
+CHECKINTIME -&gt; OrderStartTime
+CHECKOUTTIME -&gt; OrderEndTime
+DELIVERED -&gt; OrderStatus
+PACKAGING -&gt; UnitOfMeasure
+'' -&gt; Currency
+QUANTITY -&gt; QuantityOrdered
+TOTAL_VAT_INC -&gt; AmountOrdered
+DISCOUNT -&gt; Discount
+TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3325,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SHOP_ID -&gt; StoreID</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3347,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SALES_REP -&gt; SalesRepID</t>
         </is>
       </c>
     </row>
@@ -3544,7 +3369,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ROUTEID -&gt; RouteID</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3391,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>as-is (no letter strip)</t>
+          <t>PRODUCT_CODE -&gt; ProductID</t>
         </is>
       </c>
     </row>
@@ -3583,12 +3408,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(literal ???)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>constant "???"</t>
+          <t>'' -&gt; DistributorID</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3435,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SUPPLIER_ID -&gt; WarehouseID</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3457,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ENTRY_ID -&gt; OrderNumber</t>
         </is>
       </c>
     </row>
@@ -3654,7 +3479,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>CHECKINTIME -&gt; OrderDate</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3501,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>HH:mm:ss</t>
+          <t>CHECKINTIME -&gt; OrderStartTime</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3523,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>HH:mm:ss</t>
+          <t>CHECKOUTTIME -&gt; OrderEndTime</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3545,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>DELIVERED -&gt; OrderStatus</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3567,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>PACKAGING -&gt; UnitOfMeasure</t>
         </is>
       </c>
     </row>
@@ -3759,12 +3584,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>(constant)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>KES</t>
+          <t>'' -&gt; Currency</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3611,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>QUANTITY -&gt; QuantityOrdered</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3633,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>TOTAL_VAT_INC -&gt; AmountOrdered</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3655,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>DISCOUNT -&gt; Discount</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3677,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Product Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -859,129 +859,80 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="220" customHeight="1">
+    <row r="4" ht="280" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 1,
-      "productcode": "BIC502418",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502418",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "uomname": "PACKET"
-    },
-    {
-      "id": 2,
-      "productcode": "BIC502419",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "product_desc": "CRISTAL MED BLK BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502419",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "uomname": "PACKET"
-    }
-  ]
+  "id": 1,
+  "productcode": "BIC502418",
+  "product_category": "STATIONERY",
+  "product_name": "BIC",
+  "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
+  "product_status": "Enabled",
+  "short_code": "BIC502418",
+  "tax_code": "A",
+  "hs_code": null,
+  "focus_product": 0,
+  "tonne_equivalent": null,
+  "apply_discount": null,
+  "disable_price_check": false,
+  "product_type": "item",
+  "supplier": "BIC EAST AFRCA LIMITED",
+  "alternative_group": null,
+  "supplier_id": 2,
+  "uomname": "PACKET"
 }</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 1,
-      "ProductID": "502418",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502418",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "UnitofMeasure": "PACKET"
-    },
-    {
-      "id": 2,
-      "ProductID": "502419",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "ProductSKU": "CRISTAL MED BLK BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502419",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "UnitofMeasure": "PACKET"
-    }
-  ]
+  "id": 1,
+  "ProductID": "502418",
+  "product_category": "STATIONERY",
+  "product_name": "BIC",
+  "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
+  "product_status": "Enabled",
+  "short_code": "BIC502418",
+  "tax_code": "A",
+  "hs_code": "",
+  "focus_product": 0,
+  "tonne_equivalent": "",
+  "apply_discount": "",
+  "disable_price_check": false,
+  "product_type": "item",
+  "supplier": "BIC EAST AFRCA LIMITED",
+  "alternative_group": "",
+  "supplier_id": 2,
+  "UnitofMeasure": "PACKET"
 }</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>id ← id
-ProductID ← productcode  (strip leading letters (BIC502418 → 502418))
-product_category ← product_category
-product_name ← product_name
-ProductSKU ← product_desc
-product_status ← product_status
-short_code ← short_code
-tax_code ← tax_code
-hs_code ← hs_code
-focus_product ← focus_product
-tonne_equivalent ← tonne_equivalent
-apply_discount ← apply_discount
-disable_price_check ← disable_price_check
-product_type ← product_type
-supplier ← supplier
-alternative_group ← alternative_group
-supplier_id ← supplier_id
-UnitofMeasure ← uomname
-Notes: productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>id -&gt; id
+productcode -&gt; ProductID
+product_category -&gt; product_category
+product_name -&gt; product_name
+product_desc -&gt; ProductSKU
+product_status -&gt; product_status
+short_code -&gt; short_code
+tax_code -&gt; tax_code
+hs_code -&gt; hs_code
+focus_product -&gt; focus_product
+tonne_equivalent -&gt; tonne_equivalent
+apply_discount -&gt; apply_discount
+disable_price_check -&gt; disable_price_check
+product_type -&gt; product_type
+supplier -&gt; supplier
+alternative_group -&gt; alternative_group
+supplier_id -&gt; supplier_id
+uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -2045,7 +1996,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="220" customHeight="1">
+    <row r="4" ht="280" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Product</t>
@@ -2079,120 +2030,71 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 1,
-      "productcode": "BIC502418",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502418",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "uomname": "PACKET"
-    },
-    {
-      "id": 2,
-      "productcode": "BIC502419",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "product_desc": "CRISTAL MED BLK BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502419",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "uomname": "PACKET"
-    }
-  ]
+  "id": 1,
+  "productcode": "BIC502418",
+  "product_category": "STATIONERY",
+  "product_name": "BIC",
+  "product_desc": "CRISTAL MED BLU BX 25 BCL KE",
+  "product_status": "Enabled",
+  "short_code": "BIC502418",
+  "tax_code": "A",
+  "hs_code": null,
+  "focus_product": 0,
+  "tonne_equivalent": null,
+  "apply_discount": null,
+  "disable_price_check": false,
+  "product_type": "item",
+  "supplier": "BIC EAST AFRCA LIMITED",
+  "alternative_group": null,
+  "supplier_id": 2,
+  "uomname": "PACKET"
 }</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 1,
-      "ProductID": "502418",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502418",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "UnitofMeasure": "PACKET"
-    },
-    {
-      "id": 2,
-      "ProductID": "502419",
-      "product_category": "STATIONERY",
-      "product_name": "BIC",
-      "ProductSKU": "CRISTAL MED BLK BX 25 BCL KE",
-      "product_status": "Enabled",
-      "short_code": "BIC502419",
-      "tax_code": "A",
-      "hs_code": null,
-      "focus_product": 0,
-      "tonne_equivalent": null,
-      "apply_discount": null,
-      "disable_price_check": false,
-      "product_type": "item",
-      "supplier": "BIC EAST AFRCA LIMITED",
-      "alternative_group": null,
-      "supplier_id": 2,
-      "UnitofMeasure": "PACKET"
-    }
-  ]
+  "id": 1,
+  "ProductID": "502418",
+  "product_category": "STATIONERY",
+  "product_name": "BIC",
+  "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
+  "product_status": "Enabled",
+  "short_code": "BIC502418",
+  "tax_code": "A",
+  "hs_code": "",
+  "focus_product": 0,
+  "tonne_equivalent": "",
+  "apply_discount": "",
+  "disable_price_check": false,
+  "product_type": "item",
+  "supplier": "BIC EAST AFRCA LIMITED",
+  "alternative_group": "",
+  "supplier_id": 2,
+  "UnitofMeasure": "PACKET"
 }</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>id ← id
-ProductID ← productcode  (strip leading letters (BIC502418 → 502418))
-product_category ← product_category
-product_name ← product_name
-ProductSKU ← product_desc
-product_status ← product_status
-short_code ← short_code
-tax_code ← tax_code
-hs_code ← hs_code
-focus_product ← focus_product
-tonne_equivalent ← tonne_equivalent
-apply_discount ← apply_discount
-disable_price_check ← disable_price_check
-product_type ← product_type
-supplier ← supplier
-alternative_group ← alternative_group
-supplier_id ← supplier_id
-UnitofMeasure ← uomname
-productcode→ProductID (from first numeric). product_desc→ProductSKU. uomname→UnitofMeasure. One SAPI field per output field.</t>
+          <t>id -&gt; id
+productcode -&gt; ProductID
+product_category -&gt; product_category
+product_name -&gt; product_name
+product_desc -&gt; ProductSKU
+product_status -&gt; product_status
+short_code -&gt; short_code
+tax_code -&gt; tax_code
+hs_code -&gt; hs_code
+focus_product -&gt; focus_product
+tonne_equivalent -&gt; tonne_equivalent
+apply_discount -&gt; apply_discount
+disable_price_check -&gt; disable_price_check
+product_type -&gt; product_type
+supplier -&gt; supplier
+alternative_group -&gt; alternative_group
+supplier_id -&gt; supplier_id
+uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3601,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>id -&gt; id</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3623,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>strip leading letters (BIC502418 → 502418)</t>
+          <t>productcode -&gt; ProductID</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3645,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>product_category -&gt; product_category</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3667,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>product_name -&gt; product_name</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3689,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>product_desc -&gt; ProductSKU</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3711,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>product_status -&gt; product_status</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3733,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>short_code -&gt; short_code</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3755,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>tax_code -&gt; tax_code</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3777,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>hs_code -&gt; hs_code</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3799,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>focus_product -&gt; focus_product</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3821,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>tonne_equivalent -&gt; tonne_equivalent</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3843,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>apply_discount -&gt; apply_discount</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3865,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>disable_price_check -&gt; disable_price_check</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3887,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>product_type -&gt; product_type</t>
         </is>
       </c>
     </row>
@@ -4007,7 +3909,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>supplier -&gt; supplier</t>
         </is>
       </c>
     </row>
@@ -4029,7 +3931,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>alternative_group -&gt; alternative_group</t>
         </is>
       </c>
     </row>
@@ -4051,7 +3953,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>supplier_id -&gt; supplier_id</t>
         </is>
       </c>
     </row>
@@ -4073,7 +3975,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Route Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -967,83 +967,48 @@
           <t>Route</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 31,
-      "route_id": 31,
-      "region_id": 1,
-      "region_name": "NAIROBI",
-      "route_name": "DICKSON NJUE MONDAY",
-      "routestatus": "Active",
-      "created_by": "CLEMENCEA SARU",
-      "updated_by": null,
-      "created_at": "2026-06-15T11:15:47",
-      "updated_at": "2026-06-15T11:15:47",
-      "userid": 75,
-      "visit_frequency": "Weekly",
-      "visit_week": "1",
-      "visit_day": "MON",
-      "status": "Active",
-      "saler_category": "Van Sales"
-    },
-    {
-      "id": 33,
-      "route_id": 33,
-      "region_id": 1,
-      "region_name": "NAIROBI",
-      "route_name": "PHILIP DAVID TUESDAY",
-      "routestatus": "Active",
-      "created_by": "CLEMENCEA SARU",
-      "updated_by": null,
-      "created_at": "2026-06-15T11:19:06",
-      "updated_at": "2026-06-15T11:19:06",
-      "userid": 73,
-      "visit_frequency": "Weekly",
-      "visit_week": "1",
-      "visit_day": "TUE",
-      "status": "Active",
-      "saler_category": "Van Sales"
-    }
-  ]
+  "id": 31,
+  "route_id": 31,
+  "region_id": 1,
+  "region_name": "NAIROBI",
+  "route_name": "DICKSON NJUE MONDAY",
+  "routestatus": "Active",
+  "created_by": "CLEMENCEA SARU",
+  "updated_by": null,
+  "created_at": "2026-06-15T11:15:47",
+  "updated_at": "2026-06-15T11:15:47",
+  "userid": 75,
+  "visit_frequency": "Weekly",
+  "visit_week": "1",
+  "visit_day": "MON",
+  "status": "Active",
+  "saler_category": "Van Sales"
 }</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "RouteID": 31,
-      "RouteName": "DICKSON NJUE MONDAY",
-      "SalesRepID": 75,
-      "RouteType": "Weekly",
-      "SalesRepType": "Van Sales",
-      "Date": "15/06/2026"
-    },
-    {
-      "RouteID": 33,
-      "RouteName": "PHILIP DAVID TUESDAY",
-      "SalesRepID": 73,
-      "RouteType": "Weekly",
-      "SalesRepType": "Van Sales",
-      "Date": "15/06/2026"
-    }
-  ]
+  "RouteID": 31,
+  "RouteName": "DICKSON NJUE MONDAY",
+  "SalesRepID": 75,
+  "RouteType": "Weekly",
+  "SalesRepType": "Van Sales",
+  "Date": "15/06/2026"
 }</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>RouteID ← route_id
-RouteName ← route_name
-SalesRepID ← userid
-RouteType ← visit_frequency
-SalesRepType ← saler_category
-Date ← created_at  (dd/MM/yyyy)
-Notes: route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>route_id -&gt; RouteID
+route_name -&gt; RouteName
+userid -&gt; SalesRepID
+visit_frequency -&gt; RouteType
+saler_category -&gt; SalesRepType
+created_at -&gt; Date</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -2098,7 +2063,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="180" customHeight="1">
+    <row r="5" ht="220" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Route</t>
@@ -2132,80 +2097,45 @@
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 31,
-      "route_id": 31,
-      "region_id": 1,
-      "region_name": "NAIROBI",
-      "route_name": "DICKSON NJUE MONDAY",
-      "routestatus": "Active",
-      "created_by": "CLEMENCEA SARU",
-      "updated_by": null,
-      "created_at": "2026-06-15T11:15:47",
-      "updated_at": "2026-06-15T11:15:47",
-      "userid": 75,
-      "visit_frequency": "Weekly",
-      "visit_week": "1",
-      "visit_day": "MON",
-      "status": "Active",
-      "saler_category": "Van Sales"
-    },
-    {
-      "id": 33,
-      "route_id": 33,
-      "region_id": 1,
-      "region_name": "NAIROBI",
-      "route_name": "PHILIP DAVID TUESDAY",
-      "routestatus": "Active",
-      "created_by": "CLEMENCEA SARU",
-      "updated_by": null,
-      "created_at": "2026-06-15T11:19:06",
-      "updated_at": "2026-06-15T11:19:06",
-      "userid": 73,
-      "visit_frequency": "Weekly",
-      "visit_week": "1",
-      "visit_day": "TUE",
-      "status": "Active",
-      "saler_category": "Van Sales"
-    }
-  ]
+  "id": 31,
+  "route_id": 31,
+  "region_id": 1,
+  "region_name": "NAIROBI",
+  "route_name": "DICKSON NJUE MONDAY",
+  "routestatus": "Active",
+  "created_by": "CLEMENCEA SARU",
+  "updated_by": null,
+  "created_at": "2026-06-15T11:15:47",
+  "updated_at": "2026-06-15T11:15:47",
+  "userid": 75,
+  "visit_frequency": "Weekly",
+  "visit_week": "1",
+  "visit_day": "MON",
+  "status": "Active",
+  "saler_category": "Van Sales"
 }</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "RouteID": 31,
-      "RouteName": "DICKSON NJUE MONDAY",
-      "SalesRepID": 75,
-      "RouteType": "Weekly",
-      "SalesRepType": "Van Sales",
-      "Date": "15/06/2026"
-    },
-    {
-      "RouteID": 33,
-      "RouteName": "PHILIP DAVID TUESDAY",
-      "SalesRepID": 73,
-      "RouteType": "Weekly",
-      "SalesRepType": "Van Sales",
-      "Date": "15/06/2026"
-    }
-  ]
+  "RouteID": 31,
+  "RouteName": "DICKSON NJUE MONDAY",
+  "SalesRepID": 75,
+  "RouteType": "Weekly",
+  "SalesRepType": "Van Sales",
+  "Date": "15/06/2026"
 }</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>RouteID ← route_id
-RouteName ← route_name
-SalesRepID ← userid
-RouteType ← visit_frequency
-SalesRepType ← saler_category
-Date ← created_at  (dd/MM/yyyy)
-route_id, route_name, userid, visit_frequency, saler_category, created_at. Date dd/MM/yyyy. One field each.</t>
+          <t>route_id -&gt; RouteID
+route_name -&gt; RouteName
+userid -&gt; SalesRepID
+visit_frequency -&gt; RouteType
+saler_category -&gt; SalesRepType
+created_at -&gt; Date</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3927,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>route_id -&gt; RouteID</t>
         </is>
       </c>
     </row>
@@ -4019,7 +3949,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>route_name -&gt; RouteName</t>
         </is>
       </c>
     </row>
@@ -4041,7 +3971,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>userid -&gt; SalesRepID</t>
         </is>
       </c>
     </row>
@@ -4063,7 +3993,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>visit_frequency -&gt; RouteType</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4015,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>saler_category -&gt; SalesRepType</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4037,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>created_at -&gt; Date</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill SalesRep Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1043,90 +1043,51 @@
           <t>SalesRep</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 72,
-      "user_reference": null,
-      "warehouse_code": null,
-      "user_type": 2,
-      "user_channel": 1,
-      "region_id": 1,
-      "rep_category": 4,
-      "name": "ESTHER KAGIRI",
-      "email": "ngong@nobleoutlook.co.ke",
-      "phone_number": "0710000000",
-      "last_time_active": "3",
-      "trackactivities": "YES",
-      "demoaccount": "",
-      "billing": "billable",
-      "status": "Inactive",
-      "territory_id": null,
-      "rolegroup_id": 4,
-      "vehicle_id": 4,
-      "added_by": 3,
-      "created_at": "2026-06-12T06:40:33",
-      "saler_category": "Drivers (Delivery Agents)"
-    },
-    {
-      "id": 73,
-      "user_reference": null,
-      "warehouse_code": null,
-      "user_type": 2,
-      "user_channel": 1,
-      "region_id": 1,
-      "rep_category": 5,
-      "name": "PHILLIP DAVID",
-      "email": "ngong1@nobleoutlook.co.ke",
-      "phone_number": "0710000001",
-      "last_time_active": "5",
-      "trackactivities": "YES",
-      "demoaccount": "",
-      "billing": "billable",
-      "status": "Active",
-      "territory_id": null,
-      "rolegroup_id": 5,
-      "vehicle_id": 2,
-      "added_by": 3,
-      "created_at": "2026-06-12T06:44:40",
-      "saler_category": "Van Sales"
-    }
-  ]
+  "id": 72,
+  "user_reference": null,
+  "warehouse_code": null,
+  "user_type": 2,
+  "user_channel": 1,
+  "region_id": 1,
+  "rep_category": 4,
+  "name": "ESTHER KAGIRI",
+  "email": "ngong@nobleoutlook.co.ke",
+  "phone_number": "0710000000",
+  "last_time_active": "3",
+  "trackactivities": "YES",
+  "demoaccount": "",
+  "billing": "billable",
+  "status": "Inactive",
+  "territory_id": null,
+  "rolegroup_id": 4,
+  "vehicle_id": 4,
+  "added_by": 3,
+  "created_at": "2026-06-12T06:40:33",
+  "saler_category": "Drivers (Delivery Agents)"
 }</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "SalesRepID": 72,
-      "SalesRepName": "ESTHER KAGIRI",
-      "DistributorID": "???",
-      "WarehouseID": "",
-      "SalesRepType": "Drivers (Delivery Agents)"
-    },
-    {
-      "SalesRepID": 73,
-      "SalesRepName": "PHILLIP DAVID",
-      "DistributorID": "???",
-      "WarehouseID": "",
-      "SalesRepType": "Van Sales"
-    }
-  ]
+  "SalesRepID": 72,
+  "SalesRepName": "ESTHER KAGIRI",
+  "DistributorID": "???",
+  "WarehouseID": "",
+  "SalesRepType": "Drivers (Delivery Agents)"
 }</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>SalesRepID ← id
-SalesRepName ← name
-DistributorID ← (literal ???)  (constant "???")
-WarehouseID ← warehouse_code
-SalesRepType ← saler_category
-Notes: id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>id -&gt; SalesRepID
+name -&gt; SalesRepName
+'' -&gt; DistributorID
+warehouse_code -&gt; WarehouseID
+saler_category -&gt; SalesRepType</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -2139,7 +2100,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="180" customHeight="1">
+    <row r="6" ht="220" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>SalesRep</t>
@@ -2173,87 +2134,48 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "id": 72,
-      "user_reference": null,
-      "warehouse_code": null,
-      "user_type": 2,
-      "user_channel": 1,
-      "region_id": 1,
-      "rep_category": 4,
-      "name": "ESTHER KAGIRI",
-      "email": "ngong@nobleoutlook.co.ke",
-      "phone_number": "0710000000",
-      "last_time_active": "3",
-      "trackactivities": "YES",
-      "demoaccount": "",
-      "billing": "billable",
-      "status": "Inactive",
-      "territory_id": null,
-      "rolegroup_id": 4,
-      "vehicle_id": 4,
-      "added_by": 3,
-      "created_at": "2026-06-12T06:40:33",
-      "saler_category": "Drivers (Delivery Agents)"
-    },
-    {
-      "id": 73,
-      "user_reference": null,
-      "warehouse_code": null,
-      "user_type": 2,
-      "user_channel": 1,
-      "region_id": 1,
-      "rep_category": 5,
-      "name": "PHILLIP DAVID",
-      "email": "ngong1@nobleoutlook.co.ke",
-      "phone_number": "0710000001",
-      "last_time_active": "5",
-      "trackactivities": "YES",
-      "demoaccount": "",
-      "billing": "billable",
-      "status": "Active",
-      "territory_id": null,
-      "rolegroup_id": 5,
-      "vehicle_id": 2,
-      "added_by": 3,
-      "created_at": "2026-06-12T06:44:40",
-      "saler_category": "Van Sales"
-    }
-  ]
+  "id": 72,
+  "user_reference": null,
+  "warehouse_code": null,
+  "user_type": 2,
+  "user_channel": 1,
+  "region_id": 1,
+  "rep_category": 4,
+  "name": "ESTHER KAGIRI",
+  "email": "ngong@nobleoutlook.co.ke",
+  "phone_number": "0710000000",
+  "last_time_active": "3",
+  "trackactivities": "YES",
+  "demoaccount": "",
+  "billing": "billable",
+  "status": "Inactive",
+  "territory_id": null,
+  "rolegroup_id": 4,
+  "vehicle_id": 4,
+  "added_by": 3,
+  "created_at": "2026-06-12T06:40:33",
+  "saler_category": "Drivers (Delivery Agents)"
 }</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "SalesRepID": 72,
-      "SalesRepName": "ESTHER KAGIRI",
-      "DistributorID": "???",
-      "WarehouseID": "",
-      "SalesRepType": "Drivers (Delivery Agents)"
-    },
-    {
-      "SalesRepID": 73,
-      "SalesRepName": "PHILLIP DAVID",
-      "DistributorID": "???",
-      "WarehouseID": "",
-      "SalesRepType": "Van Sales"
-    }
-  ]
+  "SalesRepID": 72,
+  "SalesRepName": "ESTHER KAGIRI",
+  "DistributorID": "???",
+  "WarehouseID": "",
+  "SalesRepType": "Drivers (Delivery Agents)"
 }</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>SalesRepID ← id
-SalesRepName ← name
-DistributorID ← (literal ???)  (constant "???")
-WarehouseID ← warehouse_code
-SalesRepType ← saler_category
-id, name, warehouse_code, saler_category. DistributorID is ???. One field each.</t>
+          <t>id -&gt; SalesRepID
+name -&gt; SalesRepName
+'' -&gt; DistributorID
+warehouse_code -&gt; WarehouseID
+saler_category -&gt; SalesRepType</t>
         </is>
       </c>
     </row>
@@ -4059,7 +3981,7 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>id -&gt; SalesRepID</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4003,7 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>name -&gt; SalesRepName</t>
         </is>
       </c>
     </row>
@@ -4098,12 +4020,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>(literal ???)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>constant "???"</t>
+          <t>'' -&gt; DistributorID</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4047,7 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>warehouse_code -&gt; WarehouseID</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4069,7 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>saler_category -&gt; SalesRepType</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Customer Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1116,171 +1116,99 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="220" customHeight="1">
+    <row r="7" ht="280" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 199,
-      "SHOPID": 199,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 183,
-      "shop_cat_id": 2,
-      "shop_subcat_id": 2,
-      "CUSTOMERCODE": null,
-      "CUSTOMERNAME": "MANDELA SHOP",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 85,
-      "LOCATIONNAME": "RUIRU",
-      "CUSTOMERCATEGORY": "RETAIL SHOP",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "INDIRECT",
-      "SUPPLIER": "GIKAMBURA STOCKPOINT",
-      "PHONENUMBER": "+254722590524",
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "IAN MWENDWA",
-      "VERIFIEDDATE": "2026-06-15T14:35:26",
-      "ADDEDBY": "PHILLIP DAVID",
-      "USERID": 73,
-      "USERCATEGORY": "Van Sales",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": "PINCH ANISO",
-      "KRAPIN": null,
-      "LASTVISIT": "2026-09-07T15:27:43",
-      "LASTSALE": "2026-06-15T15:07:50",
-      "LATITUDE": -1.2349905,
-      "LONGITUDE": 36.9328219,
-      "DATECREATED": "2026-06-15T14:17:10",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Customer"
-    },
-    {
-      "ID": 200,
-      "SHOPID": 200,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 183,
-      "shop_cat_id": 2,
-      "shop_subcat_id": 2,
-      "CUSTOMERCODE": null,
-      "CUSTOMERNAME": "GB SHOP",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 85,
-      "LOCATIONNAME": "RUIRU",
-      "CUSTOMERCATEGORY": "RETAIL SHOP",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "INDIRECT",
-      "SUPPLIER": "GIKAMBURA STOCKPOINT",
-      "PHONENUMBER": "+254725446821",
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "CLEMENCEA SARU",
-      "VERIFIEDDATE": "2026-06-15T16:09:14",
-      "ADDEDBY": "DICKSON NJUE",
-      "USERID": 75,
-      "USERCATEGORY": "Van Sales",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": "GB",
-      "KRAPIN": null,
-      "LASTVISIT": "2026-09-07T15:28:04",
-      "LASTSALE": "2026-08-31T17:08:17",
-      "LATITUDE": -1.2562547,
-      "LONGITUDE": 36.9237899,
-      "DATECREATED": "2026-06-15T16:07:17",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Customer"
-    }
-  ]
+  "ID": 199,
+  "SHOPID": 199,
+  "PARENT_ID": null,
+  "region_id": 1,
+  "group_id": 0,
+  "supplied_by": 183,
+  "shop_cat_id": 2,
+  "shop_subcat_id": 2,
+  "CUSTOMERCODE": null,
+  "CUSTOMERNAME": "MANDELA SHOP",
+  "IS_HQ": "no",
+  "ACCOUNT_ID": 0,
+  "ACCOUNT": null,
+  "REGIONNAME": "NAIROBI",
+  "LOCATION_ID": 85,
+  "LOCATIONNAME": "RUIRU",
+  "CUSTOMERCATEGORY": "RETAIL SHOP",
+  "TERRITORY_NAME": null,
+  "CHANNEL": "GENERAL TRADE",
+  "RELATIONSHIP": "INDIRECT",
+  "SUPPLIER": "GIKAMBURA STOCKPOINT",
+  "PHONENUMBER": "+254722590524",
+  "VERIFIED": "Valid",
+  "VERIFIEDBY": "IAN MWENDWA",
+  "VERIFIEDDATE": "2026-06-15T14:35:26",
+  "ADDEDBY": "PHILLIP DAVID",
+  "USERID": 73,
+  "USERCATEGORY": "Van Sales",
+  "EMAILADDRESS": "",
+  "CONTACTPERSON": "PINCH ANISO",
+  "KRAPIN": null,
+  "LASTVISIT": "2026-09-07T15:27:43",
+  "LASTSALE": "2026-06-15T15:07:50",
+  "LATITUDE": -1.2349905,
+  "LONGITUDE": 36.9328219,
+  "DATECREATED": "2026-06-15T14:17:10",
+  "STATUS": 1,
+  "DISTRIBUTOR_ID": null,
+  "COUNTRY_ID": 113,
+  "COUNTRY_NAME": "KENYA",
+  "CONVERTED_LEAD": "Yes",
+  "CREDIT_LIMIT": 0,
+  "PAYMENT_TERMS": null,
+  "CREDIT_DAYS": null,
+  "CUSTOMER_TYPE": "Customer"
 }</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "StoreID": 199,
-      "StoreName": "MANDELA SHOP",
-      "StoreCategory": "RETAIL SHOP",
-      "Channel": "GENERAL TRADE",
-      "StoreClassification": "GENERAL TRADE",
-      "WarehouseID": "???",
-      "Longitude": 36.9328219,
-      "Latitude": -1.2349905,
-      "City": "RUIRU",
-      "Region": "NAIROBI",
-      "County": "",
-      "StoreStatus": 1,
-      "StoreCreationDate": "15/06/2026",
-      "StoreSize": ""
-    },
-    {
-      "StoreID": 200,
-      "StoreName": "GB SHOP",
-      "StoreCategory": "RETAIL SHOP",
-      "Channel": "GENERAL TRADE",
-      "StoreClassification": "GENERAL TRADE",
-      "WarehouseID": "???",
-      "Longitude": 36.9237899,
-      "Latitude": -1.2562547,
-      "City": "RUIRU",
-      "Region": "NAIROBI",
-      "County": "",
-      "StoreStatus": 1,
-      "StoreCreationDate": "15/06/2026",
-      "StoreSize": ""
-    }
-  ]
+  "StoreID": 199,
+  "StoreName": "MANDELA SHOP",
+  "StoreCategory": "RETAIL SHOP",
+  "Channel": "GENERAL TRADE",
+  "StoreClassification": "GENERAL TRADE",
+  "WarehouseID": "???",
+  "Longitude": 36.9328219,
+  "Latitude": -1.2349905,
+  "City": "RUIRU",
+  "Region": "NAIROBI",
+  "County": "",
+  "StoreStatus": 1,
+  "StoreCreationDate": "15/06/2026",
+  "StoreSize": ""
 }</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>StoreID ← SHOPID
-StoreName ← CUSTOMERNAME
-StoreCategory ← CUSTOMERCATEGORY
-Channel ← CHANNEL
-StoreClassification ← CHANNEL  (same as Channel)
-WarehouseID ← (literal ???)  (constant "???")
-Longitude ← LONGITUDE
-Latitude ← LATITUDE
-City ← LOCATIONNAME
-Region ← REGIONNAME
-County ← (hardcoded empty)  (constant empty)
-StoreStatus ← STATUS
-StoreCreationDate ← DATECREATED  (dd/MM/yyyy)
-StoreSize ← (hardcoded empty)  (constant empty)
-Notes: CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>SHOPID -&gt; StoreID
+CUSTOMERNAME -&gt; StoreName
+CUSTOMERCATEGORY -&gt; StoreCategory
+CHANNEL -&gt; Channel
+CHANNEL -&gt; StoreClassification
+'' -&gt; WarehouseID
+LONGITUDE -&gt; Longitude
+LATITUDE -&gt; Latitude
+LOCATIONNAME -&gt; City
+REGIONNAME -&gt; Region
+'' -&gt; County
+STATUS -&gt; StoreStatus
+DATECREATED -&gt; StoreCreationDate
+'' -&gt; StoreSize</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -2179,7 +2107,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="200" customHeight="1">
+    <row r="7" ht="280" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Customer</t>
@@ -2213,162 +2141,90 @@
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 199,
-      "SHOPID": 199,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 183,
-      "shop_cat_id": 2,
-      "shop_subcat_id": 2,
-      "CUSTOMERCODE": null,
-      "CUSTOMERNAME": "MANDELA SHOP",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 85,
-      "LOCATIONNAME": "RUIRU",
-      "CUSTOMERCATEGORY": "RETAIL SHOP",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "INDIRECT",
-      "SUPPLIER": "GIKAMBURA STOCKPOINT",
-      "PHONENUMBER": "+254722590524",
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "IAN MWENDWA",
-      "VERIFIEDDATE": "2026-06-15T14:35:26",
-      "ADDEDBY": "PHILLIP DAVID",
-      "USERID": 73,
-      "USERCATEGORY": "Van Sales",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": "PINCH ANISO",
-      "KRAPIN": null,
-      "LASTVISIT": "2026-09-07T15:27:43",
-      "LASTSALE": "2026-06-15T15:07:50",
-      "LATITUDE": -1.2349905,
-      "LONGITUDE": 36.9328219,
-      "DATECREATED": "2026-06-15T14:17:10",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Customer"
-    },
-    {
-      "ID": 200,
-      "SHOPID": 200,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 183,
-      "shop_cat_id": 2,
-      "shop_subcat_id": 2,
-      "CUSTOMERCODE": null,
-      "CUSTOMERNAME": "GB SHOP",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 85,
-      "LOCATIONNAME": "RUIRU",
-      "CUSTOMERCATEGORY": "RETAIL SHOP",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "INDIRECT",
-      "SUPPLIER": "GIKAMBURA STOCKPOINT",
-      "PHONENUMBER": "+254725446821",
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "CLEMENCEA SARU",
-      "VERIFIEDDATE": "2026-06-15T16:09:14",
-      "ADDEDBY": "DICKSON NJUE",
-      "USERID": 75,
-      "USERCATEGORY": "Van Sales",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": "GB",
-      "KRAPIN": null,
-      "LASTVISIT": "2026-09-07T15:28:04",
-      "LASTSALE": "2026-08-31T17:08:17",
-      "LATITUDE": -1.2562547,
-      "LONGITUDE": 36.9237899,
-      "DATECREATED": "2026-06-15T16:07:17",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Customer"
-    }
-  ]
+  "ID": 199,
+  "SHOPID": 199,
+  "PARENT_ID": null,
+  "region_id": 1,
+  "group_id": 0,
+  "supplied_by": 183,
+  "shop_cat_id": 2,
+  "shop_subcat_id": 2,
+  "CUSTOMERCODE": null,
+  "CUSTOMERNAME": "MANDELA SHOP",
+  "IS_HQ": "no",
+  "ACCOUNT_ID": 0,
+  "ACCOUNT": null,
+  "REGIONNAME": "NAIROBI",
+  "LOCATION_ID": 85,
+  "LOCATIONNAME": "RUIRU",
+  "CUSTOMERCATEGORY": "RETAIL SHOP",
+  "TERRITORY_NAME": null,
+  "CHANNEL": "GENERAL TRADE",
+  "RELATIONSHIP": "INDIRECT",
+  "SUPPLIER": "GIKAMBURA STOCKPOINT",
+  "PHONENUMBER": "+254722590524",
+  "VERIFIED": "Valid",
+  "VERIFIEDBY": "IAN MWENDWA",
+  "VERIFIEDDATE": "2026-06-15T14:35:26",
+  "ADDEDBY": "PHILLIP DAVID",
+  "USERID": 73,
+  "USERCATEGORY": "Van Sales",
+  "EMAILADDRESS": "",
+  "CONTACTPERSON": "PINCH ANISO",
+  "KRAPIN": null,
+  "LASTVISIT": "2026-09-07T15:27:43",
+  "LASTSALE": "2026-06-15T15:07:50",
+  "LATITUDE": -1.2349905,
+  "LONGITUDE": 36.9328219,
+  "DATECREATED": "2026-06-15T14:17:10",
+  "STATUS": 1,
+  "DISTRIBUTOR_ID": null,
+  "COUNTRY_ID": 113,
+  "COUNTRY_NAME": "KENYA",
+  "CONVERTED_LEAD": "Yes",
+  "CREDIT_LIMIT": 0,
+  "PAYMENT_TERMS": null,
+  "CREDIT_DAYS": null,
+  "CUSTOMER_TYPE": "Customer"
 }</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "StoreID": 199,
-      "StoreName": "MANDELA SHOP",
-      "StoreCategory": "RETAIL SHOP",
-      "Channel": "GENERAL TRADE",
-      "StoreClassification": "GENERAL TRADE",
-      "WarehouseID": "???",
-      "Longitude": 36.9328219,
-      "Latitude": -1.2349905,
-      "City": "RUIRU",
-      "Region": "NAIROBI",
-      "County": "",
-      "StoreStatus": 1,
-      "StoreCreationDate": "15/06/2026",
-      "StoreSize": ""
-    },
-    {
-      "StoreID": 200,
-      "StoreName": "GB SHOP",
-      "StoreCategory": "RETAIL SHOP",
-      "Channel": "GENERAL TRADE",
-      "StoreClassification": "GENERAL TRADE",
-      "WarehouseID": "???",
-      "Longitude": 36.9237899,
-      "Latitude": -1.2562547,
-      "City": "RUIRU",
-      "Region": "NAIROBI",
-      "County": "",
-      "StoreStatus": 1,
-      "StoreCreationDate": "15/06/2026",
-      "StoreSize": ""
-    }
-  ]
+  "StoreID": 199,
+  "StoreName": "MANDELA SHOP",
+  "StoreCategory": "RETAIL SHOP",
+  "Channel": "GENERAL TRADE",
+  "StoreClassification": "GENERAL TRADE",
+  "WarehouseID": "???",
+  "Longitude": 36.9328219,
+  "Latitude": -1.2349905,
+  "City": "RUIRU",
+  "Region": "NAIROBI",
+  "County": "",
+  "StoreStatus": 1,
+  "StoreCreationDate": "15/06/2026",
+  "StoreSize": ""
 }</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>StoreID ← SHOPID
-StoreName ← CUSTOMERNAME
-StoreCategory ← CUSTOMERCATEGORY
-Channel ← CHANNEL
-StoreClassification ← CHANNEL  (same as Channel)
-WarehouseID ← (literal ???)  (constant "???")
-Longitude ← LONGITUDE
-Latitude ← LATITUDE
-City ← LOCATIONNAME
-Region ← REGIONNAME
-County ← (hardcoded empty)  (constant empty)
-StoreStatus ← STATUS
-StoreCreationDate ← DATECREATED  (dd/MM/yyyy)
-StoreSize ← (hardcoded empty)  (constant empty)
-CHANNEL maps to Channel and StoreClassification. WarehouseID is ???. County and StoreSize are empty.</t>
+          <t>SHOPID -&gt; StoreID
+CUSTOMERNAME -&gt; StoreName
+CUSTOMERCATEGORY -&gt; StoreCategory
+CHANNEL -&gt; Channel
+CHANNEL -&gt; StoreClassification
+'' -&gt; WarehouseID
+LONGITUDE -&gt; Longitude
+LATITUDE -&gt; Latitude
+LOCATIONNAME -&gt; City
+REGIONNAME -&gt; Region
+'' -&gt; County
+STATUS -&gt; StoreStatus
+DATECREATED -&gt; StoreCreationDate
+'' -&gt; StoreSize</t>
         </is>
       </c>
     </row>
@@ -4091,7 +3947,7 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>SHOPID -&gt; StoreID</t>
         </is>
       </c>
     </row>
@@ -4113,7 +3969,7 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>CUSTOMERNAME -&gt; StoreName</t>
         </is>
       </c>
     </row>
@@ -4135,7 +3991,7 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>CUSTOMERCATEGORY -&gt; StoreCategory</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4013,7 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>CHANNEL -&gt; Channel</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4035,7 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>same as Channel</t>
+          <t>CHANNEL -&gt; StoreClassification</t>
         </is>
       </c>
     </row>
@@ -4196,12 +4052,12 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>(literal ???)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>constant "???"</t>
+          <t>'' -&gt; WarehouseID</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4079,7 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>LONGITUDE -&gt; Longitude</t>
         </is>
       </c>
     </row>
@@ -4245,7 +4101,7 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>LATITUDE -&gt; Latitude</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4123,7 @@
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>LOCATIONNAME -&gt; City</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4145,7 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>REGIONNAME -&gt; Region</t>
         </is>
       </c>
     </row>
@@ -4306,12 +4162,12 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>(hardcoded empty)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>constant empty</t>
+          <t>'' -&gt; County</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4189,7 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>STATUS -&gt; StoreStatus</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4211,7 @@
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>DATECREATED -&gt; StoreCreationDate</t>
         </is>
       </c>
     </row>
@@ -4372,12 +4228,12 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>(hardcoded empty)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>constant empty</t>
+          <t>'' -&gt; StoreSize</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Stock Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1237,69 +1237,44 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="220" customHeight="1">
+    <row r="8" ht="180" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "productcode": "BIC969584",
-      "uomname": "PACKET",
-      "stockpoint_name": null,
-      "date_created": "2026-08-17T14:00:56",
-      "quantity": 2640,
-      "total_cost": 1060
-    },
-    {
-      "productcode": "BIC969584",
-      "uomname": "PACKET",
-      "stockpoint_name": "GIKAMBURA STOCKPOINT",
-      "date_created": "2026-08-14T12:42:33",
-      "quantity": 2640,
-      "total_cost": 1116
-    }
-  ]
+  "productcode": "BIC969584",
+  "uomname": "PACKET",
+  "stockpoint_name": null,
+  "date_created": "2026-08-17T14:00:56",
+  "quantity": 2640,
+  "total_cost": 1060
 }</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ProductSKU": "969584",
-      "UnitofMeasure": "PACKET",
-      "DistributorWarehouseCode": "",
-      "Date": "17/08/2026",
-      "InventoryQuantity": 2640,
-      "InventoryPrice": 1060
-    },
-    {
-      "ProductSKU": "969584",
-      "UnitofMeasure": "PACKET",
-      "DistributorWarehouseCode": "GIKAMBURA STOCKPOINT",
-      "Date": "14/08/2026",
-      "InventoryQuantity": 2640,
-      "InventoryPrice": 1116
-    }
-  ]
+  "ProductSKU": "969584",
+  "UnitofMeasure": "PACKET",
+  "DistributorWarehouseCode": "",
+  "Date": "17/08/2026",
+  "InventoryQuantity": 2640,
+  "InventoryPrice": 1060
 }</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>ProductSKU ← productcode  (from first numeric (BIC969584 → 969584))
-UnitofMeasure ← uomname
-DistributorWarehouseCode ← stockpoint_name
-Date ← date_created  (dd/MM/yyyy)
-InventoryQuantity ← quantity
-InventoryPrice ← total_cost
-Notes: productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>productcode -&gt; ProductSKU
+uomname -&gt; UnitofMeasure
+stockpoint_name -&gt; DistributorWarehouseCode
+date_created -&gt; Date
+quantity -&gt; InventoryQuantity
+total_cost -&gt; InventoryPrice</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -2262,60 +2237,35 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "productcode": "BIC969584",
-      "uomname": "PACKET",
-      "stockpoint_name": null,
-      "date_created": "2026-08-17T14:00:56",
-      "quantity": 2640,
-      "total_cost": 1060
-    },
-    {
-      "productcode": "BIC969584",
-      "uomname": "PACKET",
-      "stockpoint_name": "GIKAMBURA STOCKPOINT",
-      "date_created": "2026-08-14T12:42:33",
-      "quantity": 2640,
-      "total_cost": 1116
-    }
-  ]
+  "productcode": "BIC969584",
+  "uomname": "PACKET",
+  "stockpoint_name": null,
+  "date_created": "2026-08-17T14:00:56",
+  "quantity": 2640,
+  "total_cost": 1060
 }</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ProductSKU": "969584",
-      "UnitofMeasure": "PACKET",
-      "DistributorWarehouseCode": "",
-      "Date": "17/08/2026",
-      "InventoryQuantity": 2640,
-      "InventoryPrice": 1060
-    },
-    {
-      "ProductSKU": "969584",
-      "UnitofMeasure": "PACKET",
-      "DistributorWarehouseCode": "GIKAMBURA STOCKPOINT",
-      "Date": "14/08/2026",
-      "InventoryQuantity": 2640,
-      "InventoryPrice": 1116
-    }
-  ]
+  "ProductSKU": "969584",
+  "UnitofMeasure": "PACKET",
+  "DistributorWarehouseCode": "",
+  "Date": "17/08/2026",
+  "InventoryQuantity": 2640,
+  "InventoryPrice": 1060
 }</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>ProductSKU ← productcode  (from first numeric (BIC969584 → 969584))
-UnitofMeasure ← uomname
-DistributorWarehouseCode ← stockpoint_name
-Date ← date_created  (dd/MM/yyyy)
-InventoryQuantity ← quantity
-InventoryPrice ← total_cost
-productcode→ProductSKU from first numeric. uomname, stockpoint_name, date_created, quantity, total_cost. One field each.</t>
+          <t>productcode -&gt; ProductSKU
+uomname -&gt; UnitofMeasure
+stockpoint_name -&gt; DistributorWarehouseCode
+date_created -&gt; Date
+quantity -&gt; InventoryQuantity
+total_cost -&gt; InventoryPrice</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4205,7 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>from first numeric (BIC969584 → 969584)</t>
+          <t>productcode -&gt; ProductSKU</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4227,7 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4249,7 @@
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>stockpoint_name -&gt; DistributorWarehouseCode</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4271,7 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>dd/MM/yyyy</t>
+          <t>date_created -&gt; Date</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4293,7 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>quantity -&gt; InventoryQuantity</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4315,7 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>total_cost -&gt; InventoryPrice</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Warehouse Excel from real SAPI and transformed payloads.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1303,138 +1303,77 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="220" customHeight="1">
+    <row r="9" ht="180" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Warehouse</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 183,
-      "SHOPID": 183,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 0,
-      "shop_cat_id": 1,
-      "shop_subcat_id": null,
-      "CUSTOMERCODE": "183",
-      "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 4,
-      "LOCATIONNAME": "GIKAMBURA",
-      "CUSTOMERCATEGORY": "WHOLESALE",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "DIRECT",
-      "SUPPLIER": null,
-      "PHONENUMBER": null,
-      "VERIFIED": "Pending",
-      "VERIFIEDBY": null,
-      "VERIFIEDDATE": null,
-      "ADDEDBY": "TECLA AYORE",
-      "USERID": 3,
-      "USERCATEGORY": "Admin",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": null,
-      "KRAPIN": null,
-      "LASTVISIT": null,
-      "LASTSALE": null,
-      "LATITUDE": null,
-      "LONGITUDE": null,
-      "DATECREATED": "2026-06-08T15:07:59",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Supplier"
-    },
-    {
-      "ID": 186,
-      "SHOPID": 186,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 0,
-      "shop_cat_id": 1,
-      "shop_subcat_id": null,
-      "CUSTOMERCODE": "186",
-      "CUSTOMERNAME": "NAIROBI WEST STCKPOINT",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 1,
-      "LOCATIONNAME": "NAIROBI WEST",
-      "CUSTOMERCATEGORY": "WHOLESALE",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "DIRECT",
-      "SUPPLIER": null,
-      "PHONENUMBER": null,
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "TECLA AYORE",
-      "VERIFIEDDATE": "2026-06-09T22:46:16",
-      "ADDEDBY": "TECLA AYORE",
-      "USERID": 3,
-      "USERCATEGORY": "Admin",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": null,
-      "KRAPIN": null,
-      "LASTVISIT": null,
-      "LASTSALE": null,
-      "LATITUDE": null,
-      "LONGITUDE": null,
-      "DATECREATED": "2026-06-09T22:42:10",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Supplier"
-    }
-  ]
+  "ID": 183,
+  "SHOPID": 183,
+  "PARENT_ID": null,
+  "region_id": 1,
+  "group_id": 0,
+  "supplied_by": 0,
+  "shop_cat_id": 1,
+  "shop_subcat_id": null,
+  "CUSTOMERCODE": "183",
+  "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
+  "IS_HQ": "no",
+  "ACCOUNT_ID": 0,
+  "ACCOUNT": null,
+  "REGIONNAME": "NAIROBI",
+  "LOCATION_ID": 4,
+  "LOCATIONNAME": "GIKAMBURA",
+  "CUSTOMERCATEGORY": "WHOLESALE",
+  "TERRITORY_NAME": null,
+  "CHANNEL": "GENERAL TRADE",
+  "RELATIONSHIP": "DIRECT",
+  "SUPPLIER": null,
+  "PHONENUMBER": null,
+  "VERIFIED": "Pending",
+  "VERIFIEDBY": null,
+  "VERIFIEDDATE": null,
+  "ADDEDBY": "TECLA AYORE",
+  "USERID": 3,
+  "USERCATEGORY": "Admin",
+  "EMAILADDRESS": "",
+  "CONTACTPERSON": null,
+  "KRAPIN": null,
+  "LASTVISIT": null,
+  "LASTSALE": null,
+  "LATITUDE": null,
+  "LONGITUDE": null,
+  "DATECREATED": "2026-06-08T15:07:59",
+  "STATUS": 1,
+  "DISTRIBUTOR_ID": null,
+  "COUNTRY_ID": 113,
+  "COUNTRY_NAME": "KENYA",
+  "CONVERTED_LEAD": "Yes",
+  "CREDIT_LIMIT": 0,
+  "PAYMENT_TERMS": null,
+  "CREDIT_DAYS": null,
+  "CUSTOMER_TYPE": "Supplier"
 }</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "WarehouseID": 183,
-      "WarehouseName": "GIKAMBURA STOCKPOINT",
-      "DistributorID": ""
-    },
-    {
-      "WarehouseID": 186,
-      "WarehouseName": "NAIROBI WEST STCKPOINT",
-      "DistributorID": ""
-    }
-  ]
+  "WarehouseID": 183,
+  "WarehouseName": "GIKAMBURA STOCKPOINT",
+  "DistributorID": ""
 }</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>WarehouseID ← ID
-WarehouseName ← CUSTOMERNAME
-DistributorID ← (hardcoded empty)  (constant empty)
-Notes: ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>ID -&gt; WarehouseID
+CUSTOMERNAME -&gt; WarehouseName
+'' -&gt; DistributorID</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -2303,129 +2242,68 @@
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "ID": 183,
-      "SHOPID": 183,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 0,
-      "shop_cat_id": 1,
-      "shop_subcat_id": null,
-      "CUSTOMERCODE": "183",
-      "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 4,
-      "LOCATIONNAME": "GIKAMBURA",
-      "CUSTOMERCATEGORY": "WHOLESALE",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "DIRECT",
-      "SUPPLIER": null,
-      "PHONENUMBER": null,
-      "VERIFIED": "Pending",
-      "VERIFIEDBY": null,
-      "VERIFIEDDATE": null,
-      "ADDEDBY": "TECLA AYORE",
-      "USERID": 3,
-      "USERCATEGORY": "Admin",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": null,
-      "KRAPIN": null,
-      "LASTVISIT": null,
-      "LASTSALE": null,
-      "LATITUDE": null,
-      "LONGITUDE": null,
-      "DATECREATED": "2026-06-08T15:07:59",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Supplier"
-    },
-    {
-      "ID": 186,
-      "SHOPID": 186,
-      "PARENT_ID": null,
-      "region_id": 1,
-      "group_id": 0,
-      "supplied_by": 0,
-      "shop_cat_id": 1,
-      "shop_subcat_id": null,
-      "CUSTOMERCODE": "186",
-      "CUSTOMERNAME": "NAIROBI WEST STCKPOINT",
-      "IS_HQ": "no",
-      "ACCOUNT_ID": 0,
-      "ACCOUNT": null,
-      "REGIONNAME": "NAIROBI",
-      "LOCATION_ID": 1,
-      "LOCATIONNAME": "NAIROBI WEST",
-      "CUSTOMERCATEGORY": "WHOLESALE",
-      "TERRITORY_NAME": null,
-      "CHANNEL": "GENERAL TRADE",
-      "RELATIONSHIP": "DIRECT",
-      "SUPPLIER": null,
-      "PHONENUMBER": null,
-      "VERIFIED": "Valid",
-      "VERIFIEDBY": "TECLA AYORE",
-      "VERIFIEDDATE": "2026-06-09T22:46:16",
-      "ADDEDBY": "TECLA AYORE",
-      "USERID": 3,
-      "USERCATEGORY": "Admin",
-      "EMAILADDRESS": "",
-      "CONTACTPERSON": null,
-      "KRAPIN": null,
-      "LASTVISIT": null,
-      "LASTSALE": null,
-      "LATITUDE": null,
-      "LONGITUDE": null,
-      "DATECREATED": "2026-06-09T22:42:10",
-      "STATUS": 1,
-      "DISTRIBUTOR_ID": null,
-      "COUNTRY_ID": 113,
-      "COUNTRY_NAME": "KENYA",
-      "CONVERTED_LEAD": "Yes",
-      "CREDIT_LIMIT": 0,
-      "PAYMENT_TERMS": null,
-      "CREDIT_DAYS": null,
-      "CUSTOMER_TYPE": "Supplier"
-    }
-  ]
+  "ID": 183,
+  "SHOPID": 183,
+  "PARENT_ID": null,
+  "region_id": 1,
+  "group_id": 0,
+  "supplied_by": 0,
+  "shop_cat_id": 1,
+  "shop_subcat_id": null,
+  "CUSTOMERCODE": "183",
+  "CUSTOMERNAME": "GIKAMBURA STOCKPOINT",
+  "IS_HQ": "no",
+  "ACCOUNT_ID": 0,
+  "ACCOUNT": null,
+  "REGIONNAME": "NAIROBI",
+  "LOCATION_ID": 4,
+  "LOCATIONNAME": "GIKAMBURA",
+  "CUSTOMERCATEGORY": "WHOLESALE",
+  "TERRITORY_NAME": null,
+  "CHANNEL": "GENERAL TRADE",
+  "RELATIONSHIP": "DIRECT",
+  "SUPPLIER": null,
+  "PHONENUMBER": null,
+  "VERIFIED": "Pending",
+  "VERIFIEDBY": null,
+  "VERIFIEDDATE": null,
+  "ADDEDBY": "TECLA AYORE",
+  "USERID": 3,
+  "USERCATEGORY": "Admin",
+  "EMAILADDRESS": "",
+  "CONTACTPERSON": null,
+  "KRAPIN": null,
+  "LASTVISIT": null,
+  "LASTSALE": null,
+  "LATITUDE": null,
+  "LONGITUDE": null,
+  "DATECREATED": "2026-06-08T15:07:59",
+  "STATUS": 1,
+  "DISTRIBUTOR_ID": null,
+  "COUNTRY_ID": 113,
+  "COUNTRY_NAME": "KENYA",
+  "CONVERTED_LEAD": "Yes",
+  "CREDIT_LIMIT": 0,
+  "PAYMENT_TERMS": null,
+  "CREDIT_DAYS": null,
+  "CUSTOMER_TYPE": "Supplier"
 }</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>{
-  "data": [
-    {
-      "WarehouseID": 183,
-      "WarehouseName": "GIKAMBURA STOCKPOINT",
-      "DistributorID": ""
-    },
-    {
-      "WarehouseID": 186,
-      "WarehouseName": "NAIROBI WEST STCKPOINT",
-      "DistributorID": ""
-    }
-  ]
+  "WarehouseID": 183,
+  "WarehouseName": "GIKAMBURA STOCKPOINT",
+  "DistributorID": ""
 }</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>WarehouseID ← ID
-WarehouseName ← CUSTOMERNAME
-DistributorID ← (hardcoded empty)  (constant empty)
-ID→WarehouseID, CUSTOMERNAME→WarehouseName, DistributorID empty. One field each. SAPI warehouse SQL is CUSTOMER_TYPE='Supplier'. stockpoint_id EXISTS stays commented until Solutech adds the column.</t>
+          <t>ID -&gt; WarehouseID
+CUSTOMERNAME -&gt; WarehouseName
+'' -&gt; DistributorID</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4215,7 @@
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>ID -&gt; WarehouseID</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4237,7 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>as-is</t>
+          <t>CUSTOMERNAME -&gt; WarehouseName</t>
         </is>
       </c>
     </row>
@@ -4376,12 +4254,12 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>(hardcoded empty)</t>
+          <t>''</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>constant empty</t>
+          <t>'' -&gt; DistributorID</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SAPI SQL query column for each datashare endpoint.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -142,6 +142,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -509,14 +513,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
@@ -546,25 +550,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Query</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>SAPI endpoint</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PAPI endpoint</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Exp endpoint</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>PAPI mapping file</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -692,27 +701,38 @@
 ENTRY_TYPE -&gt; TransType</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*, b.routeid
+from sat_nobleoutlook.bi_salesmaster as a
+left join sat_nobleoutlook.bi_customer_visits as b on a.VisitID = b.visitid
+inner join sat_nobleoutlook.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = 'BIC EAST AFRCA LIMITED'
+where a.Created_AT between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 00:00:00'
+order by a.Entry_ID desc
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>/api/invoice</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>/api/Adapter_Invoice</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>/api/v1/Invoice</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>dwl/map-adapter-invoice.dwl</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -833,27 +853,37 @@
 TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*, b.routeid, b.CHECKINTIME, b.CHECKOUTTIME
+from sat_nobleoutlook.bi_ordersmaster as a
+inner join sat_nobleoutlook.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = 'BIC EAST AFRCA LIMITED'
+left join sat_nobleoutlook.bi_customer_visits as b on a.VISIT_ID = b.visitid
+order by a.ENTRY_ID desc
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>/api/order</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>/api/Adapter_Order</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>/api/v1/Order</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>dwl/map-adapter-order.dwl</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -935,27 +965,38 @@
 uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*, c.uomname
+from sat_nobleoutlook.bi_products as a
+left join sat_nobleoutlook.bi_uom_quantities as b on a.id = b.product_id
+left join sat_nobleoutlook.bi_uom as c on b.packaging_id = c.id
+where a.supplier = 'BIC EAST AFRCA LIMITED'
+order by a.id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>/api/product</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>/api/Adapter_Product</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>/api/v1/Product</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>dwl/map-adapter-product.dwl</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -1011,27 +1052,54 @@
 created_at -&gt; Date</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*, b.userid, b.visit_frequency, b.visit_week, b.visit_day, b.status, d.saler_category
+from sat_nobleoutlook.bi_routes as a
+left join sat_nobleoutlook.bi_user_routes as b on a.route_id = b.route_id
+left join sat_nobleoutlook.bi_users as c on b.userid = c.id
+left join sat_nobleoutlook.bi_user_categories as d on c.rep_category = d.usercategory
+where exists (
+  Select 1 from (
+    Select distinct routeid from (
+      select Distinct v.routeid, y.product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      inner join sat_nobleoutlook.bi_customer_visits as v on y.VisitID = v.visitid
+      union all
+      select Distinct v.routeid, y.product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+      inner join sat_nobleoutlook.bi_customer_visits as v on y.Visit_ID = v.visitid
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.routeid = a.route_id
+)
+order by a.route_id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>/api/route</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>/api/Adapter_Route</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>/api/v1/Route</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>dwl/map-adapter-route.dwl</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -1090,27 +1158,50 @@
 saler_category -&gt; SalesRepType</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*, b.saler_category
+from sat_nobleoutlook.bi_users as a
+left join sat_nobleoutlook.bi_user_categories as b on a.rep_category = b.usercategory
+where exists (
+  Select 1 from (
+    Select distinct userid from (
+      select Distinct userid, y.product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      union all
+      select Distinct user_id as userid, y.product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.userid = a.id
+)
+order by a.id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>/api/sales-rep</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>/api/Adapter_SalesRep</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>/api/v1/SalesRep</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>dwl/map-adapter-salesrep.dwl</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -1211,33 +1302,56 @@
 '' -&gt; StoreSize</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Select a.*
+from sat_nobleoutlook.bi_customer_master as a
+where a.Customer_Type = 'Customer'
+and exists (
+  Select 1 from (
+    Select distinct SHOPID from (
+      select Distinct SHOPID, product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      union all
+      select Distinct SHOP_ID as SHOPID, product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.SHOPID = a.SHOPID
+)
+order by a.SHOPID
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>/api/customer</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>/api/Adapter_Customer</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>/api/v1/Customer</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>dwl/map-adapter-customer.dwl</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="180" customHeight="1">
+    <row r="8" ht="220" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Stock</t>
@@ -1277,33 +1391,46 @@
 total_cost -&gt; InventoryPrice</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Select a.productcode, d.UOMName, b.stockpoint_name, MAX(b.date_created) as date_created, SUM(b.quantity) as quantity, SUM(b.total_cost) as total_cost
+from sat_nobleoutlook.bi_products as a
+inner join sat_nobleoutlook.bi_stock_movement as b on a.id = b.product_id
+left join sat_nobleoutlook.bi_uom_quantities as c on b.product_id = c.product_id
+left join sat_nobleoutlook.bi_uom as d on c.packaging_id = d.id
+where a.supplier = 'BIC EAST AFRCA LIMITED'
+group by a.id, d.UOMName, b.stockpoint_name
+order by a.id, d.UOMName, b.stockpoint_name
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>/api/stock</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>/api/Adapter_Stock</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>/api/v1/Stock</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>dwl/map-adapter-stock.dwl</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="180" customHeight="1">
+    <row r="9" ht="220" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Warehouse</t>
@@ -1376,27 +1503,44 @@
 '' -&gt; DistributorID</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Select c.*
+from sat_nobleoutlook.bi_customer_master as c
+where CUSTOMER_TYPE = 'Supplier' /*Hardcoded value*/
+/*and exists
+Select 1
+from
+(select distinct stockpoint_id from sat_nobleoutlook.bi_products as a
+inner join sat_nobleoutlook.bi_stock_movement as b on a.id = b.product_id
+where a.supplier = 'BIC EAST AFRCA LIMITED') as z
+and z.stockpoint_id = c.id
+*/
+order by c.SHOPID
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>/api/warehouse</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>/api/Adapter_Warehouse</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>/api/v1/Warehouse</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>dwl/map-adapter-warehouse.dwl</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>DONE — mapped from real SAPI payload</t>
         </is>
@@ -1414,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1426,6 +1570,7 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1472,6 +1617,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Mapping notes</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Query</t>
         </is>
       </c>
     </row>
@@ -1622,6 +1772,17 @@
 ENTRY_TYPE -&gt; TransType</t>
         </is>
       </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*, b.routeid
+from sat_nobleoutlook.bi_salesmaster as a
+left join sat_nobleoutlook.bi_customer_visits as b on a.VisitID = b.visitid
+inner join sat_nobleoutlook.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = 'BIC EAST AFRCA LIMITED'
+where a.Created_AT between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 00:00:00'
+order by a.Entry_ID desc
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="280" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1763,6 +1924,16 @@
 TOTAL_VAT -&gt; VATAmount</t>
         </is>
       </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*, b.routeid, b.CHECKINTIME, b.CHECKOUTTIME
+from sat_nobleoutlook.bi_ordersmaster as a
+inner join sat_nobleoutlook.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = 'BIC EAST AFRCA LIMITED'
+left join sat_nobleoutlook.bi_customer_visits as b on a.VISIT_ID = b.visitid
+order by a.ENTRY_ID desc
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="280" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1865,6 +2036,17 @@
 uomname -&gt; UnitofMeasure</t>
         </is>
       </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*, c.uomname
+from sat_nobleoutlook.bi_products as a
+left join sat_nobleoutlook.bi_uom_quantities as b on a.id = b.product_id
+left join sat_nobleoutlook.bi_uom as c on b.packaging_id = c.id
+where a.supplier = 'BIC EAST AFRCA LIMITED'
+order by a.id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="220" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1939,6 +2121,33 @@
 visit_frequency -&gt; RouteType
 saler_category -&gt; SalesRepType
 created_at -&gt; Date</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*, b.userid, b.visit_frequency, b.visit_week, b.visit_day, b.status, d.saler_category
+from sat_nobleoutlook.bi_routes as a
+left join sat_nobleoutlook.bi_user_routes as b on a.route_id = b.route_id
+left join sat_nobleoutlook.bi_users as c on b.userid = c.id
+left join sat_nobleoutlook.bi_user_categories as d on c.rep_category = d.usercategory
+where exists (
+  Select 1 from (
+    Select distinct routeid from (
+      select Distinct v.routeid, y.product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      inner join sat_nobleoutlook.bi_customer_visits as v on y.VisitID = v.visitid
+      union all
+      select Distinct v.routeid, y.product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+      inner join sat_nobleoutlook.bi_customer_visits as v on y.Visit_ID = v.visitid
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.routeid = a.route_id
+)
+order by a.route_id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
       </c>
     </row>
@@ -2018,6 +2227,29 @@
 '' -&gt; DistributorID
 warehouse_code -&gt; WarehouseID
 saler_category -&gt; SalesRepType</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*, b.saler_category
+from sat_nobleoutlook.bi_users as a
+left join sat_nobleoutlook.bi_user_categories as b on a.rep_category = b.usercategory
+where exists (
+  Select 1 from (
+    Select distinct userid from (
+      select Distinct userid, y.product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      union all
+      select Distinct user_id as userid, y.product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.userid = a.id
+)
+order by a.id
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
       </c>
     </row>
@@ -2141,6 +2373,29 @@
 '' -&gt; StoreSize</t>
         </is>
       </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Select a.*
+from sat_nobleoutlook.bi_customer_master as a
+where a.Customer_Type = 'Customer'
+and exists (
+  Select 1 from (
+    Select distinct SHOPID from (
+      select Distinct SHOPID, product_id
+      from sat_nobleoutlook.bi_salesmaster as y
+      union all
+      select Distinct SHOP_ID as SHOPID, product_id
+      from sat_nobleoutlook.bi_ordersmaster as y
+    ) as x
+    inner join sat_nobleoutlook.bi_products as z on x.product_id = z.id
+    where z.supplier = 'BIC EAST AFRCA LIMITED'
+  ) as w
+  where w.SHOPID = a.SHOPID
+)
+order by a.SHOPID
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="180" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -2205,6 +2460,19 @@
 date_created -&gt; Date
 quantity -&gt; InventoryQuantity
 total_cost -&gt; InventoryPrice</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Select a.productcode, d.UOMName, b.stockpoint_name, MAX(b.date_created) as date_created, SUM(b.quantity) as quantity, SUM(b.total_cost) as total_cost
+from sat_nobleoutlook.bi_products as a
+inner join sat_nobleoutlook.bi_stock_movement as b on a.id = b.product_id
+left join sat_nobleoutlook.bi_uom_quantities as c on b.product_id = c.product_id
+left join sat_nobleoutlook.bi_uom as d on c.packaging_id = d.id
+where a.supplier = 'BIC EAST AFRCA LIMITED'
+group by a.id, d.UOMName, b.stockpoint_name
+order by a.id, d.UOMName, b.stockpoint_name
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
       </c>
     </row>
@@ -2306,6 +2574,23 @@
 '' -&gt; DistributorID</t>
         </is>
       </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Select c.*
+from sat_nobleoutlook.bi_customer_master as c
+where CUSTOMER_TYPE = 'Supplier' /*Hardcoded value*/
+/*and exists
+Select 1
+from
+(select distinct stockpoint_id from sat_nobleoutlook.bi_products as a
+inner join sat_nobleoutlook.bi_stock_movement as b on a.id = b.product_id
+where a.supplier = 'BIC EAST AFRCA LIMITED') as z
+and z.stockpoint_id = c.id
+*/
+order by c.SHOPID
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>